<commit_message>
chore: update geo-ip data - 20250912_133152
📊 Data sync summary:
- Updated at: 2025-09-12 13:31:54 UTC
- Territories: 250
- IP ranges: 258299
- Data size: 41.20MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-08-12T03:16:22.102Z</t>
+    <t>2025-09-12T13:30:06.263Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 256807</t>
+    <t>Total IP ranges: 258299</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>256807</v>
+        <v>258299</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1859</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7238</v>
+        <v>7251</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2313</v>
+        <v>2322</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>1973</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4930</v>
+        <v>5035</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4802</v>
+        <v>4790</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8788</v>
+        <v>8731</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4903,7 +4903,7 @@
         <v>44</v>
       </c>
       <c r="I42">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1014</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4422</v>
+        <v>4444</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1039</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>293</v>
+        <v>286</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1883</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1601</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>465</v>
+        <v>448</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>298</v>
+        <v>310</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>658</v>
+        <v>676</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1845</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8795</v>
+        <v>8769</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>14968</v>
+        <v>15357</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>685</v>
+        <v>695</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6500</v>
+        <v>6759</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>937</v>
+        <v>922</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7778</v>
+        <v>7714</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4407</v>
+        <v>4474</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1605</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2220</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1178</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>4977</v>
+        <v>5032</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6570</v>
+        <v>6603</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>893</v>
+        <v>907</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>894</v>
+        <v>857</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>554</v>
+        <v>545</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1433</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1611</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>287</v>
+        <v>294</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10776</v>
+        <v>10629</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1504</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>507</v>
+        <v>522</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1657</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>841</v>
+        <v>847</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>325</v>
+        <v>316</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1451</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4916</v>
+        <v>4923</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>649</v>
+        <v>661</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>374</v>
+        <v>357</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2469</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>8996</v>
+        <v>9089</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>885</v>
+        <v>920</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>574</v>
+        <v>578</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>336</v>
+        <v>296</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>63</v>
+        <v>53</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>4872</v>
+        <v>4906</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>593</v>
+        <v>594</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>574</v>
+        <v>603</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9601,7 +9601,7 @@
         <v>25</v>
       </c>
       <c r="I204">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2316</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2275</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5118</v>
+        <v>5255</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3697</v>
+        <v>3645</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3398</v>
+        <v>3444</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1400</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1249</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2380</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3578</v>
+        <v>3571</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>989</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15847</v>
+        <v>15894</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41313</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>277</v>
+        <v>288</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>475</v>
+        <v>489</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1340</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41313</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15847</v>
+        <v>15894</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>14968</v>
+        <v>15357</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10776</v>
+        <v>10629</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>777</v>
       </c>
       <c r="B17">
-        <v>8996</v>
+        <v>9089</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>8795</v>
+        <v>8769</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8788</v>
+        <v>8731</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7778</v>
+        <v>7714</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7238</v>
+        <v>7251</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>497</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>6570</v>
+        <v>6759</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20250912_144025
📊 Data sync summary:
- Updated at: 2025-09-12 14:40:28 UTC
- Territories: 250
- IP ranges: 258299
- Data size: 41.20MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-08-12T03:16:22.102Z</t>
+    <t>2025-09-12T14:38:36.962Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 256807</t>
+    <t>Total IP ranges: 258299</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>256807</v>
+        <v>258299</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1859</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7238</v>
+        <v>7251</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2313</v>
+        <v>2322</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>1973</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4930</v>
+        <v>5035</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4802</v>
+        <v>4790</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8788</v>
+        <v>8731</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4903,7 +4903,7 @@
         <v>44</v>
       </c>
       <c r="I42">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1014</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4422</v>
+        <v>4444</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1039</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>293</v>
+        <v>286</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1883</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1601</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>465</v>
+        <v>448</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>298</v>
+        <v>310</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>658</v>
+        <v>676</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1845</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8795</v>
+        <v>8769</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>14968</v>
+        <v>15357</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>685</v>
+        <v>695</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6500</v>
+        <v>6759</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>937</v>
+        <v>922</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7778</v>
+        <v>7714</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4407</v>
+        <v>4474</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1605</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2220</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1178</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>4977</v>
+        <v>5032</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6570</v>
+        <v>6603</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>893</v>
+        <v>907</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>894</v>
+        <v>857</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>554</v>
+        <v>545</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1433</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1611</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>287</v>
+        <v>294</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10776</v>
+        <v>10629</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1504</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>507</v>
+        <v>522</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1657</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>841</v>
+        <v>847</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>325</v>
+        <v>316</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1451</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4916</v>
+        <v>4923</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>649</v>
+        <v>661</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>374</v>
+        <v>357</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2469</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>8996</v>
+        <v>9089</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>885</v>
+        <v>920</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>574</v>
+        <v>578</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>336</v>
+        <v>296</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>63</v>
+        <v>53</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>4872</v>
+        <v>4906</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>593</v>
+        <v>594</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>574</v>
+        <v>603</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9601,7 +9601,7 @@
         <v>25</v>
       </c>
       <c r="I204">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2316</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2275</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5118</v>
+        <v>5255</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3697</v>
+        <v>3645</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3398</v>
+        <v>3444</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1400</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1249</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2380</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3578</v>
+        <v>3571</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>989</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15847</v>
+        <v>15894</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41313</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>277</v>
+        <v>288</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>475</v>
+        <v>489</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1340</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41313</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15847</v>
+        <v>15894</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>14968</v>
+        <v>15357</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10776</v>
+        <v>10629</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>777</v>
       </c>
       <c r="B17">
-        <v>8996</v>
+        <v>9089</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>8795</v>
+        <v>8769</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8788</v>
+        <v>8731</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7778</v>
+        <v>7714</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7238</v>
+        <v>7251</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>497</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>6570</v>
+        <v>6759</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20250912_144743
📊 Data sync summary:
- Updated at: 2025-09-12 14:47:45 UTC
- Territories: 250
- IP ranges: 258299
- Data size: 41.20MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-08-12T03:16:22.102Z</t>
+    <t>2025-09-12T14:45:57.445Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 256807</t>
+    <t>Total IP ranges: 258299</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>256807</v>
+        <v>258299</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1859</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7238</v>
+        <v>7251</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2313</v>
+        <v>2322</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>1973</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4930</v>
+        <v>5035</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4802</v>
+        <v>4790</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8788</v>
+        <v>8731</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4903,7 +4903,7 @@
         <v>44</v>
       </c>
       <c r="I42">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1014</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4422</v>
+        <v>4444</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1039</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>293</v>
+        <v>286</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1883</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1601</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>465</v>
+        <v>448</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>298</v>
+        <v>310</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>658</v>
+        <v>676</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1845</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8795</v>
+        <v>8769</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>14968</v>
+        <v>15357</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>685</v>
+        <v>695</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6500</v>
+        <v>6759</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>937</v>
+        <v>922</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7778</v>
+        <v>7714</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4407</v>
+        <v>4474</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1605</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2220</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1178</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>4977</v>
+        <v>5032</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6570</v>
+        <v>6603</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>893</v>
+        <v>907</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>894</v>
+        <v>857</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>554</v>
+        <v>545</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1433</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1611</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>287</v>
+        <v>294</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10776</v>
+        <v>10629</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1504</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>507</v>
+        <v>522</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1657</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>841</v>
+        <v>847</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>325</v>
+        <v>316</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1451</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4916</v>
+        <v>4923</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>649</v>
+        <v>661</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>374</v>
+        <v>357</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2469</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>8996</v>
+        <v>9089</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>885</v>
+        <v>920</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>574</v>
+        <v>578</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>336</v>
+        <v>296</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>63</v>
+        <v>53</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>4872</v>
+        <v>4906</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>593</v>
+        <v>594</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>574</v>
+        <v>603</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9601,7 +9601,7 @@
         <v>25</v>
       </c>
       <c r="I204">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2316</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2275</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5118</v>
+        <v>5255</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3697</v>
+        <v>3645</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3398</v>
+        <v>3444</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1400</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1249</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2380</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3578</v>
+        <v>3571</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>989</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15847</v>
+        <v>15894</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41313</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>277</v>
+        <v>288</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>475</v>
+        <v>489</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1340</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41313</v>
+        <v>41554</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15847</v>
+        <v>15894</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>14968</v>
+        <v>15357</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10776</v>
+        <v>10629</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>777</v>
       </c>
       <c r="B17">
-        <v>8996</v>
+        <v>9089</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>8795</v>
+        <v>8769</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8788</v>
+        <v>8731</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7778</v>
+        <v>7714</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7238</v>
+        <v>7251</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>497</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>6570</v>
+        <v>6759</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20250915_030832
📊 Data sync summary:
- Updated at: 2025-09-15 03:08:34 UTC
- Territories: 250
- IP ranges: 259497
- Data size: 41.39MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-09-14T03:01:30.993Z</t>
+    <t>2025-09-15T03:06:44.680Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 258299</t>
+    <t>Total IP ranges: 259497</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>258299</v>
+        <v>259497</v>
       </c>
     </row>
   </sheetData>
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1850</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7251</v>
+        <v>7367</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2322</v>
+        <v>2324</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>221</v>
+        <v>229</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>1978</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5035</v>
+        <v>5092</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4790</v>
+        <v>4803</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1391</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>364</v>
+        <v>369</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8731</v>
+        <v>8736</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1043</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4444</v>
+        <v>4424</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1021</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>286</v>
+        <v>294</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>342</v>
+        <v>335</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1876</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1729</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>413</v>
+        <v>397</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>676</v>
+        <v>672</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1886</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8769</v>
+        <v>8815</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15357</v>
+        <v>15496</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>695</v>
+        <v>688</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>212</v>
+        <v>219</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6759</v>
+        <v>6823</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>922</v>
+        <v>914</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7714</v>
+        <v>7758</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4474</v>
+        <v>4496</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1624</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2077</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1218</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5032</v>
+        <v>5065</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6603</v>
+        <v>6650</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>907</v>
+        <v>912</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>492</v>
+        <v>498</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>109</v>
+        <v>100</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>857</v>
+        <v>866</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>545</v>
+        <v>553</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1517</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1640</v>
+        <v>1642</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>498</v>
+        <v>506</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>294</v>
+        <v>288</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10629</v>
+        <v>10727</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1527</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>522</v>
+        <v>517</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1676</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>847</v>
+        <v>850</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>602</v>
+        <v>616</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1477</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4923</v>
+        <v>4880</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>357</v>
+        <v>363</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2426</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9089</v>
+        <v>9104</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>920</v>
+        <v>913</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>578</v>
+        <v>586</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>4906</v>
+        <v>5021</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>594</v>
+        <v>597</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>603</v>
+        <v>587</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9601,7 +9601,7 @@
         <v>25</v>
       </c>
       <c r="I204">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2098</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2374</v>
+        <v>2350</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5255</v>
+        <v>5274</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3645</v>
+        <v>3678</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3444</v>
+        <v>3472</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1425</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1250</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2418</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3571</v>
+        <v>3560</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1028</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15894</v>
+        <v>15825</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41554</v>
+        <v>41839</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1390</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41554</v>
+        <v>41839</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15894</v>
+        <v>15825</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15357</v>
+        <v>15496</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10629</v>
+        <v>10727</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>777</v>
       </c>
       <c r="B17">
-        <v>9089</v>
+        <v>9104</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>8769</v>
+        <v>8815</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8731</v>
+        <v>8736</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7714</v>
+        <v>7758</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7251</v>
+        <v>7367</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>445</v>
       </c>
       <c r="B22">
-        <v>6759</v>
+        <v>6823</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20251001_031219
📊 Data sync summary:
- Updated at: 2025-10-01 03:12:22 UTC
- Territories: 250
- IP ranges: 258315
- Data size: 41.20MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-09-30T02:57:59.870Z</t>
+    <t>2025-10-01T03:10:32.273Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 259497</t>
+    <t>Total IP ranges: 258315</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>259497</v>
+        <v>258315</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1868</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7367</v>
+        <v>7230</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2324</v>
+        <v>2349</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>229</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>1987</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5092</v>
+        <v>4906</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4803</v>
+        <v>4847</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1396</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8736</v>
+        <v>8271</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1053</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4424</v>
+        <v>4384</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1033</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>294</v>
+        <v>286</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1892</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1727</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>397</v>
+        <v>402</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>448</v>
+        <v>456</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1866</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8815</v>
+        <v>8844</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15496</v>
+        <v>15252</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>688</v>
+        <v>717</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>228</v>
+        <v>236</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6823</v>
+        <v>6930</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>914</v>
+        <v>923</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7758</v>
+        <v>7709</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4496</v>
+        <v>4469</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1623</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2089</v>
+        <v>2044</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1187</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5065</v>
+        <v>5137</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6650</v>
+        <v>6694</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>912</v>
+        <v>917</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>498</v>
+        <v>492</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>866</v>
+        <v>932</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1496</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1642</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>287</v>
+        <v>295</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10727</v>
+        <v>10606</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1517</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>517</v>
+        <v>531</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8412,7 +8412,7 @@
         <v>44</v>
       </c>
       <c r="I163">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1658</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>850</v>
+        <v>844</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>616</v>
+        <v>631</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1489</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>660</v>
+        <v>784</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2456</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9104</v>
+        <v>9096</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>72</v>
+        <v>54</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>913</v>
+        <v>915</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>586</v>
+        <v>592</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>294</v>
+        <v>299</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5021</v>
+        <v>5190</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>597</v>
+        <v>590</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>587</v>
+        <v>590</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2159</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2350</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5274</v>
+        <v>5193</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3678</v>
+        <v>3646</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3472</v>
+        <v>3386</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1459</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1294</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10210,7 +10210,7 @@
         <v>44</v>
       </c>
       <c r="I225">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2419</v>
+        <v>2397</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3560</v>
+        <v>3510</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15825</v>
+        <v>15920</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41839</v>
+        <v>41640</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>293</v>
+        <v>288</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>490</v>
+        <v>475</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1380</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41839</v>
+        <v>41640</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15825</v>
+        <v>15920</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15496</v>
+        <v>15252</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10727</v>
+        <v>10606</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>777</v>
       </c>
       <c r="B17">
-        <v>9104</v>
+        <v>9096</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>8815</v>
+        <v>8844</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8736</v>
+        <v>8271</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7758</v>
+        <v>7709</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7367</v>
+        <v>7230</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>445</v>
       </c>
       <c r="B22">
-        <v>6823</v>
+        <v>6930</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20251015_030608
📊 Data sync summary:
- Updated at: 2025-10-15 03:06:11 UTC
- Territories: 250
- IP ranges: 257826
- Data size: 41.12MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-10-14T03:00:16.693Z</t>
+    <t>2025-10-15T03:04:20.947Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 258315</t>
+    <t>Total IP ranges: 257826</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>258315</v>
+        <v>257826</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>262</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1857</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7230</v>
+        <v>7199</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2349</v>
+        <v>2341</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2002</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4906</v>
+        <v>4611</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4847</v>
+        <v>4797</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1406</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8271</v>
+        <v>8251</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4384</v>
+        <v>4411</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1061</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>286</v>
+        <v>299</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>405</v>
+        <v>411</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>338</v>
+        <v>342</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1848</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1720</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>402</v>
+        <v>408</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>456</v>
+        <v>459</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>674</v>
+        <v>681</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1848</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8844</v>
+        <v>8976</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15252</v>
+        <v>15337</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>717</v>
+        <v>706</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6930</v>
+        <v>7059</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>923</v>
+        <v>924</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7709</v>
+        <v>7805</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4469</v>
+        <v>4480</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1625</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2044</v>
+        <v>2075</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1181</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5137</v>
+        <v>5007</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6694</v>
+        <v>6579</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>182</v>
+        <v>170</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>917</v>
+        <v>921</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>492</v>
+        <v>506</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>932</v>
+        <v>928</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1477</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1661</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>507</v>
+        <v>500</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10606</v>
+        <v>10699</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1516</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>531</v>
+        <v>516</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1659</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>844</v>
+        <v>841</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>327</v>
+        <v>316</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1466</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4880</v>
+        <v>4933</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>784</v>
+        <v>811</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2469</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9096</v>
+        <v>9103</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>915</v>
+        <v>897</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>592</v>
+        <v>589</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5190</v>
+        <v>5079</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>590</v>
+        <v>601</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>590</v>
+        <v>584</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9601,7 +9601,7 @@
         <v>25</v>
       </c>
       <c r="I204">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2089</v>
+        <v>2079</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2293</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5193</v>
+        <v>5297</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3646</v>
+        <v>3701</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3386</v>
+        <v>3378</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10007,7 +10007,7 @@
         <v>25</v>
       </c>
       <c r="I218">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1443</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1297</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2397</v>
+        <v>2394</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3510</v>
+        <v>3521</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1015</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15920</v>
+        <v>15893</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41640</v>
+        <v>41033</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>475</v>
+        <v>481</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1379</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10848,7 +10848,7 @@
         <v>44</v>
       </c>
       <c r="I247">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="248" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41640</v>
+        <v>41033</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15920</v>
+        <v>15893</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15252</v>
+        <v>15337</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10606</v>
+        <v>10699</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>777</v>
       </c>
       <c r="B17">
-        <v>9096</v>
+        <v>9103</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>8844</v>
+        <v>8976</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8271</v>
+        <v>8251</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7709</v>
+        <v>7805</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7230</v>
+        <v>7199</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>445</v>
       </c>
       <c r="B22">
-        <v>6930</v>
+        <v>7059</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20251101_031310
📊 Data sync summary:
- Updated at: 2025-11-01 03:13:12 UTC
- Territories: 250
- IP ranges: 258426
- Data size: 41.22MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-10-31T03:10:29.759Z</t>
+    <t>2025-11-01T03:11:19.493Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 257826</t>
+    <t>Total IP ranges: 258426</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>257826</v>
+        <v>258426</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>272</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1862</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7199</v>
+        <v>7324</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2341</v>
+        <v>2370</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2006</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4611</v>
+        <v>4701</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4797</v>
+        <v>4828</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1418</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>366</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8251</v>
+        <v>8214</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1046</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4411</v>
+        <v>4389</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1054</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>299</v>
+        <v>291</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>411</v>
+        <v>404</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1868</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1730</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>408</v>
+        <v>401</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>310</v>
+        <v>305</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>681</v>
+        <v>670</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1771</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8976</v>
+        <v>8882</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15337</v>
+        <v>15175</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>706</v>
+        <v>722</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7059</v>
+        <v>7101</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>924</v>
+        <v>925</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7805</v>
+        <v>7767</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4480</v>
+        <v>4496</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1606</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2075</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1206</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5007</v>
+        <v>5020</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6579</v>
+        <v>6585</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>921</v>
+        <v>913</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>661</v>
+        <v>667</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>928</v>
+        <v>893</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>556</v>
+        <v>548</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1500</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1711</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>500</v>
+        <v>492</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10699</v>
+        <v>10857</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1507</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>516</v>
+        <v>538</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1652</v>
+        <v>1647</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>841</v>
+        <v>864</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>628</v>
+        <v>632</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1497</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4933</v>
+        <v>4910</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>811</v>
+        <v>785</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>366</v>
+        <v>360</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>154</v>
+        <v>164</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2463</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9103</v>
+        <v>9106</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>897</v>
+        <v>914</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5079</v>
+        <v>5083</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>601</v>
+        <v>583</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>584</v>
+        <v>601</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9601,7 +9601,7 @@
         <v>25</v>
       </c>
       <c r="I204">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2079</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2285</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5297</v>
+        <v>5323</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3701</v>
+        <v>3508</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3378</v>
+        <v>3379</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1453</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>222</v>
+        <v>230</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1319</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2394</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3521</v>
+        <v>3506</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1010</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15893</v>
+        <v>15824</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41033</v>
+        <v>41457</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>285</v>
+        <v>293</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1380</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10848,7 +10848,7 @@
         <v>44</v>
       </c>
       <c r="I247">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41033</v>
+        <v>41457</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15893</v>
+        <v>15824</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15337</v>
+        <v>15175</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10699</v>
+        <v>10857</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>777</v>
       </c>
       <c r="B17">
-        <v>9103</v>
+        <v>9106</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>8976</v>
+        <v>8882</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8251</v>
+        <v>8214</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7805</v>
+        <v>7767</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7199</v>
+        <v>7324</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>445</v>
       </c>
       <c r="B22">
-        <v>7059</v>
+        <v>7101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20251115_030830
📊 Data sync summary:
- Updated at: 2025-11-15 03:08:33 UTC
- Territories: 250
- IP ranges: 260421
- Data size: 41.54MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-11-14T03:13:11.956Z</t>
+    <t>2025-11-15T03:06:43.429Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 258426</t>
+    <t>Total IP ranges: 260421</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>258426</v>
+        <v>260421</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1879</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7324</v>
+        <v>7371</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2370</v>
+        <v>2357</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4701</v>
+        <v>4682</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4828</v>
+        <v>4917</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1411</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8214</v>
+        <v>8323</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4903,7 +4903,7 @@
         <v>44</v>
       </c>
       <c r="I42">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1072</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4389</v>
+        <v>4392</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1059</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>345</v>
+        <v>353</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1896</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1752</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>401</v>
+        <v>422</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>305</v>
+        <v>320</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>670</v>
+        <v>679</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1854</v>
+        <v>1859</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8882</v>
+        <v>9228</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15175</v>
+        <v>15211</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>722</v>
+        <v>718</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>234</v>
+        <v>246</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7101</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>925</v>
+        <v>944</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7767</v>
+        <v>7839</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4496</v>
+        <v>4513</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1613</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2036</v>
+        <v>2117</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1250</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5020</v>
+        <v>5053</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6585</v>
+        <v>6688</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>170</v>
+        <v>177</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>913</v>
+        <v>921</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>667</v>
+        <v>677</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>118</v>
+        <v>104</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>893</v>
+        <v>885</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>548</v>
+        <v>567</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1480</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1758</v>
+        <v>1715</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>492</v>
+        <v>501</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10857</v>
+        <v>10914</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1542</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>538</v>
+        <v>518</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1647</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>864</v>
+        <v>869</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>318</v>
+        <v>309</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4910</v>
+        <v>4995</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>785</v>
+        <v>792</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>164</v>
+        <v>172</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2380</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9106</v>
+        <v>9155</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>914</v>
+        <v>935</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5083</v>
+        <v>5107</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>583</v>
+        <v>596</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2104</v>
+        <v>2129</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2279</v>
+        <v>2254</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5323</v>
+        <v>5341</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3508</v>
+        <v>3615</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3379</v>
+        <v>3387</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1467</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1343</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2417</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3506</v>
+        <v>3526</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1015</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15824</v>
+        <v>15713</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41457</v>
+        <v>41985</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>479</v>
+        <v>473</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1366</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41457</v>
+        <v>41985</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15824</v>
+        <v>15713</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15175</v>
+        <v>15211</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,23 +11135,23 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10857</v>
+        <v>10914</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B17">
-        <v>9106</v>
+        <v>9228</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>352</v>
+        <v>777</v>
       </c>
       <c r="B18">
-        <v>8882</v>
+        <v>9155</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8214</v>
+        <v>8323</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7767</v>
+        <v>7839</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7324</v>
+        <v>7371</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>445</v>
       </c>
       <c r="B22">
-        <v>7101</v>
+        <v>7140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20251201_035250
📊 Data sync summary:
- Updated at: 2025-12-01 03:52:53 UTC
- Territories: 250
- IP ranges: 269279
- Data size: 42.92MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2025-11-30T03:26:55.161Z</t>
+    <t>2025-12-01T03:51:02.197Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 260421</t>
+    <t>Total IP ranges: 269279</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>260421</v>
+        <v>269279</v>
       </c>
     </row>
   </sheetData>
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1867</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7371</v>
+        <v>7234</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2357</v>
+        <v>2341</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2012</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4682</v>
+        <v>4729</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4917</v>
+        <v>7158</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1398</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8323</v>
+        <v>8326</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1063</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4392</v>
+        <v>4415</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1060</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>403</v>
+        <v>428</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>353</v>
+        <v>359</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1907</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1744</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>456</v>
+        <v>467</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>320</v>
+        <v>309</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>679</v>
+        <v>680</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1859</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9228</v>
+        <v>9327</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15211</v>
+        <v>15341</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>718</v>
+        <v>705</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7140</v>
+        <v>6836</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7839</v>
+        <v>7828</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4513</v>
+        <v>4542</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1609</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>389</v>
+        <v>383</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2117</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1237</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5053</v>
+        <v>5196</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6688</v>
+        <v>6768</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>921</v>
+        <v>933</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>677</v>
+        <v>687</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>885</v>
+        <v>887</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>567</v>
+        <v>561</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1485</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1715</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>501</v>
+        <v>514</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>10914</v>
+        <v>11194</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1534</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>518</v>
+        <v>516</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>145</v>
+        <v>152</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1686</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>869</v>
+        <v>871</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>309</v>
+        <v>321</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>632</v>
+        <v>916</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1492</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>4995</v>
+        <v>5008</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>792</v>
+        <v>824</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2402</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9155</v>
+        <v>9202</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>935</v>
+        <v>939</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>296</v>
+        <v>329</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5107</v>
+        <v>5187</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>596</v>
+        <v>589</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>599</v>
+        <v>593</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2129</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2254</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5341</v>
+        <v>7712</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3615</v>
+        <v>3656</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3387</v>
+        <v>3402</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -10007,7 +10007,7 @@
         <v>25</v>
       </c>
       <c r="I218">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1480</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1347</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2457</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3526</v>
+        <v>3581</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1020</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15713</v>
+        <v>16035</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>41985</v>
+        <v>44481</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>297</v>
+        <v>309</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>473</v>
+        <v>479</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1393</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>41985</v>
+        <v>44481</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15713</v>
+        <v>16035</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15211</v>
+        <v>15341</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>10914</v>
+        <v>11194</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>352</v>
       </c>
       <c r="B17">
-        <v>9228</v>
+        <v>9327</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>777</v>
       </c>
       <c r="B18">
-        <v>9155</v>
+        <v>9202</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8323</v>
+        <v>8326</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7839</v>
+        <v>7828</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>885</v>
       </c>
       <c r="B21">
-        <v>7371</v>
+        <v>7712</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>87</v>
       </c>
       <c r="B22">
-        <v>7140</v>
+        <v>7234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260111_035222
📊 Data sync summary:
- Updated at: 2026-01-11 03:52:24 UTC
- Territories: 250
- IP ranges: 262706
- Data size: 41.90MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-01-10T03:24:09.047Z</t>
+    <t>2026-01-11T03:50:32.498Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 269279</t>
+    <t>Total IP ranges: 262706</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>269279</v>
+        <v>262706</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1881</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7234</v>
+        <v>7260</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2341</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2026</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4729</v>
+        <v>4784</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>7158</v>
+        <v>4856</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1394</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8326</v>
+        <v>8382</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1059</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4415</v>
+        <v>4412</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1080</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>295</v>
+        <v>300</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>428</v>
+        <v>410</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>359</v>
+        <v>366</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1894</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1750</v>
+        <v>1656</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>680</v>
+        <v>728</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1892</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9327</v>
+        <v>8910</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>320</v>
+        <v>332</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15341</v>
+        <v>15349</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6836</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>944</v>
+        <v>946</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7828</v>
+        <v>7882</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4542</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1606</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2053</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1268</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5196</v>
+        <v>5155</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6768</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>933</v>
+        <v>952</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>506</v>
+        <v>527</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>96</v>
+        <v>112</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>887</v>
+        <v>867</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>561</v>
+        <v>558</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1719</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>514</v>
+        <v>488</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>44</v>
+        <v>66</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11194</v>
+        <v>11345</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1550</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>516</v>
+        <v>521</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8383,7 +8383,7 @@
         <v>44</v>
       </c>
       <c r="I162">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1653</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>871</v>
+        <v>896</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>321</v>
+        <v>300</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>916</v>
+        <v>653</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1494</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5008</v>
+        <v>5054</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>824</v>
+        <v>801</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>364</v>
+        <v>371</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>164</v>
+        <v>171</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2410</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9202</v>
+        <v>9175</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>939</v>
+        <v>955</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>591</v>
+        <v>602</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5187</v>
+        <v>5633</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>589</v>
+        <v>597</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>593</v>
+        <v>599</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2300</v>
+        <v>2307</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2278</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>7712</v>
+        <v>5375</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3656</v>
+        <v>3504</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3402</v>
+        <v>3415</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1497</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1361</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2462</v>
+        <v>2448</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3581</v>
+        <v>3629</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1067</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16035</v>
+        <v>15816</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>44481</v>
+        <v>42159</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>479</v>
+        <v>471</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1389</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>44481</v>
+        <v>42159</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>16035</v>
+        <v>15816</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15341</v>
+        <v>15349</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,23 +11135,23 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11194</v>
+        <v>11345</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>352</v>
+        <v>777</v>
       </c>
       <c r="B17">
-        <v>9327</v>
+        <v>9175</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B18">
-        <v>9202</v>
+        <v>8910</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8326</v>
+        <v>8382</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7828</v>
+        <v>7882</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>885</v>
+        <v>87</v>
       </c>
       <c r="B21">
-        <v>7712</v>
+        <v>7260</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>7234</v>
+        <v>7000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260112_035102
📊 Data sync summary:
- Updated at: 2026-01-12 03:51:04 UTC
- Territories: 250
- IP ranges: 269279
- Data size: 42.92MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-01-11T03:50:32.498Z</t>
+    <t>2026-01-12T03:49:14.863Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 262706</t>
+    <t>Total IP ranges: 269279</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>262706</v>
+        <v>269279</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1886</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7260</v>
+        <v>7234</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2340</v>
+        <v>2341</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2046</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4784</v>
+        <v>4729</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>85</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4856</v>
+        <v>7158</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1399</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8382</v>
+        <v>8326</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1067</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4412</v>
+        <v>4415</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1105</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>410</v>
+        <v>428</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>366</v>
+        <v>359</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1907</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1656</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>728</v>
+        <v>680</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1764</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8910</v>
+        <v>9327</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>332</v>
+        <v>320</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15349</v>
+        <v>15341</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>199</v>
+        <v>187</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7000</v>
+        <v>6836</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>946</v>
+        <v>944</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7882</v>
+        <v>7828</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4590</v>
+        <v>4542</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1600</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2093</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1321</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5155</v>
+        <v>5196</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6932</v>
+        <v>6768</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>172</v>
+        <v>183</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>952</v>
+        <v>933</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>527</v>
+        <v>506</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>112</v>
+        <v>96</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>867</v>
+        <v>887</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>558</v>
+        <v>561</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1741</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>488</v>
+        <v>514</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>66</v>
+        <v>44</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>295</v>
+        <v>289</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11345</v>
+        <v>11194</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1526</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>521</v>
+        <v>516</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8383,7 +8383,7 @@
         <v>44</v>
       </c>
       <c r="I162">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1673</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>896</v>
+        <v>871</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>300</v>
+        <v>321</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>653</v>
+        <v>916</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1496</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5054</v>
+        <v>5008</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>801</v>
+        <v>824</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>371</v>
+        <v>364</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2428</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9175</v>
+        <v>9202</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>955</v>
+        <v>939</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>602</v>
+        <v>591</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5633</v>
+        <v>5187</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>597</v>
+        <v>589</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>599</v>
+        <v>593</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2307</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2259</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5375</v>
+        <v>7712</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>121</v>
+        <v>107</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3504</v>
+        <v>3656</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3415</v>
+        <v>3402</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1489</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1366</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2448</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3629</v>
+        <v>3581</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1153</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15816</v>
+        <v>16035</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>42159</v>
+        <v>44481</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>317</v>
+        <v>309</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>471</v>
+        <v>479</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1400</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>42159</v>
+        <v>44481</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15816</v>
+        <v>16035</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15349</v>
+        <v>15341</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,23 +11135,23 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11345</v>
+        <v>11194</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B17">
-        <v>9175</v>
+        <v>9327</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>352</v>
+        <v>777</v>
       </c>
       <c r="B18">
-        <v>8910</v>
+        <v>9202</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8382</v>
+        <v>8326</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7882</v>
+        <v>7828</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>885</v>
       </c>
       <c r="B21">
-        <v>7260</v>
+        <v>7712</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>87</v>
       </c>
       <c r="B22">
-        <v>7000</v>
+        <v>7234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260114_034913
📊 Data sync summary:
- Updated at: 2026-01-14 03:49:15 UTC
- Territories: 250
- IP ranges: 262706
- Data size: 41.90MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-01-13T03:28:15.356Z</t>
+    <t>2026-01-14T03:47:23.120Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 269279</t>
+    <t>Total IP ranges: 262706</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>269279</v>
+        <v>262706</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1881</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7234</v>
+        <v>7260</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2341</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2026</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4729</v>
+        <v>4784</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>7158</v>
+        <v>4856</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1394</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8326</v>
+        <v>8382</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1059</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4415</v>
+        <v>4412</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1080</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>295</v>
+        <v>300</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>428</v>
+        <v>410</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>359</v>
+        <v>366</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1894</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1750</v>
+        <v>1656</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>680</v>
+        <v>728</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1892</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9327</v>
+        <v>8910</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>320</v>
+        <v>332</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15341</v>
+        <v>15349</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6836</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>944</v>
+        <v>946</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7828</v>
+        <v>7882</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4542</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1606</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2053</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1268</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5196</v>
+        <v>5155</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6768</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>933</v>
+        <v>952</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>506</v>
+        <v>527</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>96</v>
+        <v>112</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>887</v>
+        <v>867</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>561</v>
+        <v>558</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1719</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>514</v>
+        <v>488</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>44</v>
+        <v>66</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11194</v>
+        <v>11345</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1550</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>516</v>
+        <v>521</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8383,7 +8383,7 @@
         <v>44</v>
       </c>
       <c r="I162">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1653</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>871</v>
+        <v>896</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>321</v>
+        <v>300</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>916</v>
+        <v>653</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1494</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5008</v>
+        <v>5054</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>824</v>
+        <v>801</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>364</v>
+        <v>371</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>164</v>
+        <v>171</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2410</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9202</v>
+        <v>9175</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>939</v>
+        <v>955</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>591</v>
+        <v>602</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5187</v>
+        <v>5633</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>589</v>
+        <v>597</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>593</v>
+        <v>599</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2300</v>
+        <v>2307</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2278</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>7712</v>
+        <v>5375</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3656</v>
+        <v>3504</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3402</v>
+        <v>3415</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1497</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1361</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2462</v>
+        <v>2448</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3581</v>
+        <v>3629</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1067</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16035</v>
+        <v>15816</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>44481</v>
+        <v>42159</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>479</v>
+        <v>471</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1389</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>44481</v>
+        <v>42159</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>16035</v>
+        <v>15816</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15341</v>
+        <v>15349</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,23 +11135,23 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11194</v>
+        <v>11345</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>352</v>
+        <v>777</v>
       </c>
       <c r="B17">
-        <v>9327</v>
+        <v>9175</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B18">
-        <v>9202</v>
+        <v>8910</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8326</v>
+        <v>8382</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7828</v>
+        <v>7882</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>885</v>
+        <v>87</v>
       </c>
       <c r="B21">
-        <v>7712</v>
+        <v>7260</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>7234</v>
+        <v>7000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260115_034250
📊 Data sync summary:
- Updated at: 2026-01-15 03:42:52 UTC
- Territories: 250
- IP ranges: 269279
- Data size: 42.92MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-01-14T03:47:23.120Z</t>
+    <t>2026-01-15T03:41:02.887Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 262706</t>
+    <t>Total IP ranges: 269279</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>262706</v>
+        <v>269279</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1886</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7260</v>
+        <v>7234</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2340</v>
+        <v>2341</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2046</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4784</v>
+        <v>4729</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>85</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4856</v>
+        <v>7158</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1399</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8382</v>
+        <v>8326</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1067</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4412</v>
+        <v>4415</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1105</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>410</v>
+        <v>428</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>366</v>
+        <v>359</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1907</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1656</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>728</v>
+        <v>680</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1764</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>8910</v>
+        <v>9327</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>332</v>
+        <v>320</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15349</v>
+        <v>15341</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>199</v>
+        <v>187</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7000</v>
+        <v>6836</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>946</v>
+        <v>944</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7882</v>
+        <v>7828</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4590</v>
+        <v>4542</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1600</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2093</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1321</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5155</v>
+        <v>5196</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6932</v>
+        <v>6768</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>172</v>
+        <v>183</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>952</v>
+        <v>933</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>527</v>
+        <v>506</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>112</v>
+        <v>96</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>867</v>
+        <v>887</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>558</v>
+        <v>561</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1741</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>488</v>
+        <v>514</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>66</v>
+        <v>44</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>295</v>
+        <v>289</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11345</v>
+        <v>11194</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1526</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>521</v>
+        <v>516</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8383,7 +8383,7 @@
         <v>44</v>
       </c>
       <c r="I162">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1673</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>896</v>
+        <v>871</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>300</v>
+        <v>321</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>653</v>
+        <v>916</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1496</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5054</v>
+        <v>5008</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>801</v>
+        <v>824</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>371</v>
+        <v>364</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2428</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9175</v>
+        <v>9202</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>955</v>
+        <v>939</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>602</v>
+        <v>591</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5633</v>
+        <v>5187</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>597</v>
+        <v>589</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>599</v>
+        <v>593</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2307</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2259</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5375</v>
+        <v>7712</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>121</v>
+        <v>107</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3504</v>
+        <v>3656</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3415</v>
+        <v>3402</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1489</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1366</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2448</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3629</v>
+        <v>3581</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1153</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15816</v>
+        <v>16035</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>42159</v>
+        <v>44481</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>317</v>
+        <v>309</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>471</v>
+        <v>479</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1400</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>42159</v>
+        <v>44481</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>15816</v>
+        <v>16035</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15349</v>
+        <v>15341</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,23 +11135,23 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11345</v>
+        <v>11194</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B17">
-        <v>9175</v>
+        <v>9327</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>352</v>
+        <v>777</v>
       </c>
       <c r="B18">
-        <v>8910</v>
+        <v>9202</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>8382</v>
+        <v>8326</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7882</v>
+        <v>7828</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>885</v>
       </c>
       <c r="B21">
-        <v>7260</v>
+        <v>7712</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>87</v>
       </c>
       <c r="B22">
-        <v>7000</v>
+        <v>7234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260116_033247
📊 Data sync summary:
- Updated at: 2026-01-16 03:32:51 UTC
- Territories: 250
- IP ranges: 267515
- Data size: 42.67MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-01-15T03:41:02.887Z</t>
+    <t>2026-01-16T03:30:49.270Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 269279</t>
+    <t>Total IP ranges: 267515</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>269279</v>
+        <v>267515</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>77</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1881</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7234</v>
+        <v>7187</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2341</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2026</v>
+        <v>2055</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4729</v>
+        <v>5239</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>151</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>83</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>7158</v>
+        <v>4884</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1394</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8326</v>
+        <v>9897</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1059</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4415</v>
+        <v>4463</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1080</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>428</v>
+        <v>421</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1894</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1750</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>420</v>
+        <v>416</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>309</v>
+        <v>294</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>680</v>
+        <v>709</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1892</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9327</v>
+        <v>9273</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15341</v>
+        <v>15409</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6836</v>
+        <v>7672</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>944</v>
+        <v>913</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7828</v>
+        <v>7833</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4542</v>
+        <v>4554</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1606</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2053</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1268</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5196</v>
+        <v>5129</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6768</v>
+        <v>7735</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>933</v>
+        <v>962</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>506</v>
+        <v>530</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>191</v>
+        <v>200</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>887</v>
+        <v>904</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>561</v>
+        <v>566</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1536</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1719</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>514</v>
+        <v>473</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>130</v>
+        <v>148</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11194</v>
+        <v>11384</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1550</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>516</v>
+        <v>512</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8383,7 +8383,7 @@
         <v>44</v>
       </c>
       <c r="I162">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1653</v>
+        <v>1656</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>871</v>
+        <v>876</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>321</v>
+        <v>265</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>916</v>
+        <v>636</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1494</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5008</v>
+        <v>5027</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>824</v>
+        <v>755</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2410</v>
+        <v>2362</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9202</v>
+        <v>9153</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>939</v>
+        <v>951</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5187</v>
+        <v>5671</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>589</v>
+        <v>578</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>593</v>
+        <v>594</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9601,7 +9601,7 @@
         <v>25</v>
       </c>
       <c r="I204">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2300</v>
+        <v>2335</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2278</v>
+        <v>2243</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>7712</v>
+        <v>5403</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>107</v>
+        <v>120</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3656</v>
+        <v>3507</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3402</v>
+        <v>3456</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1497</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>228</v>
+        <v>217</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1361</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>66</v>
+        <v>80</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2462</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3581</v>
+        <v>3663</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1067</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16035</v>
+        <v>15841</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>44481</v>
+        <v>43238</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1389</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>44481</v>
+        <v>43238</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>16035</v>
+        <v>15841</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>15341</v>
+        <v>15409</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,31 +11135,31 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11194</v>
+        <v>11384</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>352</v>
+        <v>201</v>
       </c>
       <c r="B17">
-        <v>9327</v>
+        <v>9897</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B18">
-        <v>9202</v>
+        <v>9273</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>201</v>
+        <v>777</v>
       </c>
       <c r="B19">
-        <v>8326</v>
+        <v>9153</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7828</v>
+        <v>7833</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>885</v>
+        <v>497</v>
       </c>
       <c r="B21">
-        <v>7712</v>
+        <v>7735</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>7234</v>
+        <v>7672</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260202_042652
📊 Data sync summary:
- Updated at: 2026-02-02 04:26:54 UTC
- Territories: 250
- IP ranges: 269235
- Data size: 42.94MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-01-31T04:06:08.263Z</t>
+    <t>2026-02-02T04:25:05.946Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 267515</t>
+    <t>Total IP ranges: 269235</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>267515</v>
+        <v>269235</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1885</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4062,7 +4062,7 @@
         <v>44</v>
       </c>
       <c r="I13">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7187</v>
+        <v>7259</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2316</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2055</v>
+        <v>2085</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5239</v>
+        <v>5534</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>127</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4884</v>
+        <v>4942</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1388</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9897</v>
+        <v>9260</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1067</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4463</v>
+        <v>4505</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1100</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>295</v>
+        <v>310</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>421</v>
+        <v>429</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>363</v>
+        <v>377</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1902</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1644</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>294</v>
+        <v>311</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>709</v>
+        <v>687</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1775</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9273</v>
+        <v>9421</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>325</v>
+        <v>330</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>15409</v>
+        <v>16259</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>188</v>
+        <v>199</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>705</v>
+        <v>717</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7672</v>
+        <v>7597</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>913</v>
+        <v>953</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>204</v>
+        <v>215</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7833</v>
+        <v>7957</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4554</v>
+        <v>4689</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1602</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2147</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1394</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5129</v>
+        <v>5160</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7735</v>
+        <v>6974</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>530</v>
+        <v>512</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>687</v>
+        <v>707</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>904</v>
+        <v>881</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>566</v>
+        <v>563</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1527</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>155</v>
+        <v>176</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1784</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>473</v>
+        <v>479</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>148</v>
+        <v>131</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>295</v>
+        <v>305</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11384</v>
+        <v>11278</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1511</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>512</v>
+        <v>523</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1656</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>876</v>
+        <v>869</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>265</v>
+        <v>317</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>636</v>
+        <v>640</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1455</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5027</v>
+        <v>5052</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>755</v>
+        <v>769</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2362</v>
+        <v>2413</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9153</v>
+        <v>9191</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>951</v>
+        <v>953</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>593</v>
+        <v>598</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>326</v>
+        <v>312</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5671</v>
+        <v>5766</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>578</v>
+        <v>598</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>594</v>
+        <v>608</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2335</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2243</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5403</v>
+        <v>5389</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>120</v>
+        <v>111</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3507</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3456</v>
+        <v>3482</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1503</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>217</v>
+        <v>232</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1381</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2427</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3663</v>
+        <v>3653</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1184</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15841</v>
+        <v>16025</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43238</v>
+        <v>43664</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>481</v>
+        <v>474</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1387</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,23 +11111,23 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43238</v>
+        <v>43664</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>989</v>
+        <v>380</v>
       </c>
       <c r="B14">
-        <v>15841</v>
+        <v>16259</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>380</v>
+        <v>989</v>
       </c>
       <c r="B15">
-        <v>15409</v>
+        <v>16025</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,23 +11135,23 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11384</v>
+        <v>11278</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>201</v>
+        <v>352</v>
       </c>
       <c r="B17">
-        <v>9897</v>
+        <v>9421</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>352</v>
+        <v>201</v>
       </c>
       <c r="B18">
-        <v>9273</v>
+        <v>9260</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>777</v>
       </c>
       <c r="B19">
-        <v>9153</v>
+        <v>9191</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7833</v>
+        <v>7957</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>497</v>
+        <v>445</v>
       </c>
       <c r="B21">
-        <v>7735</v>
+        <v>7597</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>87</v>
       </c>
       <c r="B22">
-        <v>7672</v>
+        <v>7259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260215_042456
📊 Data sync summary:
- Updated at: 2026-02-15 04:24:58 UTC
- Territories: 250
- IP ranges: 268375
- Data size: 42.80MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-02-14T04:11:17.923Z</t>
+    <t>2026-02-15T04:23:07.966Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 269235</t>
+    <t>Total IP ranges: 268375</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>269235</v>
+        <v>268375</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1901</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7259</v>
+        <v>7220</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2385</v>
+        <v>2315</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2085</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5534</v>
+        <v>5148</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4942</v>
+        <v>4997</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1405</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9260</v>
+        <v>9287</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1087</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4505</v>
+        <v>4501</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1105</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>310</v>
+        <v>356</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>429</v>
+        <v>412</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1938</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1668</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>424</v>
+        <v>429</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1774</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9421</v>
+        <v>9397</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16259</v>
+        <v>16134</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>717</v>
+        <v>726</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7597</v>
+        <v>7574</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>953</v>
+        <v>932</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7957</v>
+        <v>7977</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4689</v>
+        <v>4670</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1607</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2077</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1353</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5160</v>
+        <v>5216</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6974</v>
+        <v>6847</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>962</v>
+        <v>966</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>707</v>
+        <v>701</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>881</v>
+        <v>883</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1492</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1812</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>479</v>
+        <v>492</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>305</v>
+        <v>300</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11278</v>
+        <v>11292</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1522</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>523</v>
+        <v>518</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1670</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>640</v>
+        <v>675</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1528</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5052</v>
+        <v>5082</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>769</v>
+        <v>758</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>365</v>
+        <v>374</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2413</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9191</v>
+        <v>9213</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>953</v>
+        <v>960</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5766</v>
+        <v>5948</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>598</v>
+        <v>587</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>608</v>
+        <v>597</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2390</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2279</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5389</v>
+        <v>5527</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3534</v>
+        <v>3514</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3482</v>
+        <v>3459</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1514</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1417</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10210,7 +10210,7 @@
         <v>44</v>
       </c>
       <c r="I225">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2512</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3653</v>
+        <v>3679</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1232</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16025</v>
+        <v>15991</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43664</v>
+        <v>43154</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1414</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43664</v>
+        <v>43154</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>380</v>
       </c>
       <c r="B14">
-        <v>16259</v>
+        <v>16134</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>989</v>
       </c>
       <c r="B15">
-        <v>16025</v>
+        <v>15991</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11278</v>
+        <v>11292</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>352</v>
       </c>
       <c r="B17">
-        <v>9421</v>
+        <v>9397</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>201</v>
       </c>
       <c r="B18">
-        <v>9260</v>
+        <v>9287</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>777</v>
       </c>
       <c r="B19">
-        <v>9191</v>
+        <v>9213</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>7957</v>
+        <v>7977</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>445</v>
       </c>
       <c r="B21">
-        <v>7597</v>
+        <v>7574</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>87</v>
       </c>
       <c r="B22">
-        <v>7259</v>
+        <v>7220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260301_042508
📊 Data sync summary:
- Updated at: 2026-03-01 04:25:11 UTC
- Territories: 250
- IP ranges: 314594
- Data size: 50.04MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-02-28T03:55:06.399Z</t>
+    <t>2026-03-01T04:23:21.523Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 268375</t>
+    <t>Total IP ranges: 314594</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>268375</v>
+        <v>314594</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>286</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3917,7 +3917,7 @@
         <v>44</v>
       </c>
       <c r="I8">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1885</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4062,7 +4062,7 @@
         <v>44</v>
       </c>
       <c r="I13">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7220</v>
+        <v>7202</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2315</v>
+        <v>2321</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2110</v>
+        <v>2099</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5148</v>
+        <v>27549</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4997</v>
+        <v>4920</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1410</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9287</v>
+        <v>9326</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1061</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4501</v>
+        <v>4514</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1098</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>412</v>
+        <v>406</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1926</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1662</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>686</v>
+        <v>689</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1791</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9397</v>
+        <v>9445</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16134</v>
+        <v>16303</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>726</v>
+        <v>739</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>70</v>
+        <v>95</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>237</v>
+        <v>249</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7574</v>
+        <v>7711</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>932</v>
+        <v>938</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7977</v>
+        <v>7952</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4670</v>
+        <v>4641</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1613</v>
+        <v>1622</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2110</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1332</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5216</v>
+        <v>5282</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6847</v>
+        <v>7038</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>966</v>
+        <v>972</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>701</v>
+        <v>707</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>883</v>
+        <v>854</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1505</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1796</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>58</v>
+        <v>49</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11292</v>
+        <v>11328</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1529</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>518</v>
+        <v>524</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>869</v>
+        <v>884</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>314</v>
+        <v>309</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>675</v>
+        <v>666</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1505</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5082</v>
+        <v>5105</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>758</v>
+        <v>752</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>164</v>
+        <v>172</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2432</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9213</v>
+        <v>9241</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9224,7 +9224,7 @@
         <v>44</v>
       </c>
       <c r="I191">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>960</v>
+        <v>948</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>309</v>
+        <v>371</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5948</v>
+        <v>6216</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>587</v>
+        <v>583</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2406</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2291</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5527</v>
+        <v>5430</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>111</v>
+        <v>124</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3514</v>
+        <v>3489</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3459</v>
+        <v>3484</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1512</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2471</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3679</v>
+        <v>3686</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1220</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>15991</v>
+        <v>16117</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43154</v>
+        <v>65757</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1404</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -11111,79 +11111,79 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43154</v>
+        <v>65757</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>380</v>
+        <v>122</v>
       </c>
       <c r="B14">
-        <v>16134</v>
+        <v>27549</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>989</v>
+        <v>380</v>
       </c>
       <c r="B15">
-        <v>15991</v>
+        <v>16303</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>669</v>
+        <v>989</v>
       </c>
       <c r="B16">
-        <v>11292</v>
+        <v>16117</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>352</v>
+        <v>669</v>
       </c>
       <c r="B17">
-        <v>9397</v>
+        <v>11328</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>352</v>
       </c>
       <c r="B18">
-        <v>9287</v>
+        <v>9445</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>777</v>
+        <v>201</v>
       </c>
       <c r="B19">
-        <v>9213</v>
+        <v>9326</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>457</v>
+        <v>777</v>
       </c>
       <c r="B20">
-        <v>7977</v>
+        <v>9241</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="B21">
-        <v>7574</v>
+        <v>7952</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>7220</v>
+        <v>7711</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260315_043532
📊 Data sync summary:
- Updated at: 2026-03-15 04:35:34 UTC
- Territories: 250
- IP ranges: 271209
- Data size: 43.26MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-03-14T04:12:30.830Z</t>
+    <t>2026-03-15T04:33:42.680Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 314594</t>
+    <t>Total IP ranges: 271209</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>314594</v>
+        <v>271209</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1891</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7202</v>
+        <v>7254</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2321</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2099</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>27549</v>
+        <v>5282</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>4920</v>
+        <v>5136</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1403</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9326</v>
+        <v>9389</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1062</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4514</v>
+        <v>4518</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1115</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1932</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1660</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>306</v>
+        <v>301</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>689</v>
+        <v>706</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1798</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9445</v>
+        <v>9414</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16303</v>
+        <v>16347</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>739</v>
+        <v>733</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>249</v>
+        <v>242</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7711</v>
+        <v>7699</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>938</v>
+        <v>964</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>7952</v>
+        <v>8002</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4641</v>
+        <v>4683</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1622</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>391</v>
+        <v>397</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2126</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1369</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5282</v>
+        <v>5136</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7038</v>
+        <v>6992</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>972</v>
+        <v>970</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>515</v>
+        <v>523</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>191</v>
+        <v>198</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>707</v>
+        <v>715</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>854</v>
+        <v>865</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>568</v>
+        <v>586</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1501</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1802</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>494</v>
+        <v>489</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11328</v>
+        <v>11448</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1538</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>524</v>
+        <v>534</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1658</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>884</v>
+        <v>892</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>666</v>
+        <v>673</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1509</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5105</v>
+        <v>5098</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>752</v>
+        <v>743</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2451</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9241</v>
+        <v>9248</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>948</v>
+        <v>969</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>371</v>
+        <v>359</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>6216</v>
+        <v>6271</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>583</v>
+        <v>594</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>598</v>
+        <v>610</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2427</v>
+        <v>2382</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2336</v>
+        <v>2343</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5430</v>
+        <v>5448</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>124</v>
+        <v>109</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3489</v>
+        <v>3531</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3484</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1495</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1395</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2487</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3686</v>
+        <v>3697</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1213</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16117</v>
+        <v>16042</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>65757</v>
+        <v>43736</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10732,7 +10732,7 @@
         <v>25</v>
       </c>
       <c r="I243">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>476</v>
+        <v>489</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1398</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -11111,79 +11111,79 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>65757</v>
+        <v>43736</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>122</v>
+        <v>380</v>
       </c>
       <c r="B14">
-        <v>27549</v>
+        <v>16347</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>380</v>
+        <v>989</v>
       </c>
       <c r="B15">
-        <v>16303</v>
+        <v>16042</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>989</v>
+        <v>669</v>
       </c>
       <c r="B16">
-        <v>16117</v>
+        <v>11448</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>669</v>
+        <v>352</v>
       </c>
       <c r="B17">
-        <v>11328</v>
+        <v>9414</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>352</v>
+        <v>201</v>
       </c>
       <c r="B18">
-        <v>9445</v>
+        <v>9389</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>201</v>
+        <v>777</v>
       </c>
       <c r="B19">
-        <v>9326</v>
+        <v>9248</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>777</v>
+        <v>457</v>
       </c>
       <c r="B20">
-        <v>9241</v>
+        <v>8002</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>457</v>
+        <v>445</v>
       </c>
       <c r="B21">
-        <v>7952</v>
+        <v>7699</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>87</v>
       </c>
       <c r="B22">
-        <v>7711</v>
+        <v>7254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260401_044955
📊 Data sync summary:
- Updated at: 2026-04-01 04:49:58 UTC
- Territories: 250
- IP ranges: 273356
- Data size: 43.60MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-03-31T04:37:24.870Z</t>
+    <t>2026-04-01T04:48:06.843Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 271209</t>
+    <t>Total IP ranges: 273356</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>271209</v>
+        <v>273356</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1887</v>
+        <v>1919</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7254</v>
+        <v>7445</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2390</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2104</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5282</v>
+        <v>5232</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5136</v>
+        <v>5120</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1425</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9389</v>
+        <v>9665</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1069</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4518</v>
+        <v>4427</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1121</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>357</v>
+        <v>339</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>408</v>
+        <v>420</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1939</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1669</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>53</v>
+        <v>24</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>433</v>
+        <v>443</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>468</v>
+        <v>475</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>301</v>
+        <v>312</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1842</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9414</v>
+        <v>9198</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16347</v>
+        <v>16380</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>202</v>
+        <v>193</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>733</v>
+        <v>739</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>242</v>
+        <v>249</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7699</v>
+        <v>6887</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>964</v>
+        <v>961</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>216</v>
+        <v>221</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8002</v>
+        <v>8331</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1626</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2220</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1354</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5136</v>
+        <v>5219</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6992</v>
+        <v>6933</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>173</v>
+        <v>182</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>970</v>
+        <v>983</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>523</v>
+        <v>542</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>715</v>
+        <v>719</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>865</v>
+        <v>860</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>586</v>
+        <v>576</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1547</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>177</v>
+        <v>191</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1814</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>77</v>
+        <v>89</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11448</v>
+        <v>12227</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1549</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1678</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>892</v>
+        <v>900</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>310</v>
+        <v>302</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>673</v>
+        <v>666</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1495</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5098</v>
+        <v>5159</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>743</v>
+        <v>757</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>373</v>
+        <v>367</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>171</v>
+        <v>182</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2436</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9248</v>
+        <v>9271</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>969</v>
+        <v>960</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>597</v>
+        <v>601</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>6271</v>
+        <v>5724</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>594</v>
+        <v>615</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>610</v>
+        <v>615</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2382</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2343</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5448</v>
+        <v>5527</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3531</v>
+        <v>3662</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3534</v>
+        <v>3515</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1500</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1393</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2490</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3697</v>
+        <v>3672</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1219</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16042</v>
+        <v>16578</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43736</v>
+        <v>44892</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1411</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,23 +11111,23 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43736</v>
+        <v>44892</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>380</v>
+        <v>989</v>
       </c>
       <c r="B14">
-        <v>16347</v>
+        <v>16578</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>989</v>
+        <v>380</v>
       </c>
       <c r="B15">
-        <v>16042</v>
+        <v>16380</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,31 +11135,31 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11448</v>
+        <v>12227</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>352</v>
+        <v>201</v>
       </c>
       <c r="B17">
-        <v>9414</v>
+        <v>9665</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>777</v>
       </c>
       <c r="B18">
-        <v>9389</v>
+        <v>9271</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B19">
-        <v>9248</v>
+        <v>9198</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,23 +11167,23 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8002</v>
+        <v>8331</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>445</v>
+        <v>87</v>
       </c>
       <c r="B21">
-        <v>7699</v>
+        <v>7445</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>497</v>
       </c>
       <c r="B22">
-        <v>7254</v>
+        <v>6933</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260415_031217
📊 Data sync summary:
- Updated at: 2026-04-15 03:12:20 UTC
- Territories: 250
- IP ranges: 274896
- Data size: 43.85MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-04-14T04:46:31.480Z</t>
+    <t>2026-04-15T03:10:25.860Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 273356</t>
+    <t>Total IP ranges: 274896</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>273356</v>
+        <v>274896</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1919</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7445</v>
+        <v>7452</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2352</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2114</v>
+        <v>2123</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5232</v>
+        <v>5263</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5120</v>
+        <v>5152</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1413</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>379</v>
+        <v>384</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9665</v>
+        <v>9703</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1078</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4427</v>
+        <v>4437</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1135</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>373</v>
+        <v>395</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1955</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1667</v>
+        <v>1685</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>443</v>
+        <v>446</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>705</v>
+        <v>702</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1888</v>
+        <v>1942</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9198</v>
+        <v>9238</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16380</v>
+        <v>16444</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>193</v>
+        <v>201</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>739</v>
+        <v>749</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6887</v>
+        <v>7062</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>961</v>
+        <v>964</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8331</v>
+        <v>8377</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4683</v>
+        <v>4729</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1625</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2170</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1313</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5219</v>
+        <v>5184</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6933</v>
+        <v>6926</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>983</v>
+        <v>991</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>542</v>
+        <v>524</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>719</v>
+        <v>725</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>103</v>
+        <v>114</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>860</v>
+        <v>893</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>576</v>
+        <v>582</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1549</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1830</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>488</v>
+        <v>499</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>89</v>
+        <v>102</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>132</v>
+        <v>145</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12227</v>
+        <v>12203</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1557</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>145</v>
+        <v>154</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1743</v>
+        <v>1761</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>900</v>
+        <v>921</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>666</v>
+        <v>673</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1499</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8818,7 +8818,7 @@
         <v>44</v>
       </c>
       <c r="I177">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5159</v>
+        <v>5127</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>757</v>
+        <v>774</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2435</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9271</v>
+        <v>9292</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>960</v>
+        <v>982</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>601</v>
+        <v>609</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5724</v>
+        <v>5695</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>615</v>
+        <v>594</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>615</v>
+        <v>610</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2376</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2340</v>
+        <v>2338</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5527</v>
+        <v>5521</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3662</v>
+        <v>3676</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3515</v>
+        <v>3530</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1527</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1414</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2501</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3672</v>
+        <v>3653</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1246</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16578</v>
+        <v>16719</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>44892</v>
+        <v>45256</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1405</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>44892</v>
+        <v>45256</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>16578</v>
+        <v>16719</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>16380</v>
+        <v>16444</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12227</v>
+        <v>12203</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>201</v>
       </c>
       <c r="B17">
-        <v>9665</v>
+        <v>9703</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>777</v>
       </c>
       <c r="B18">
-        <v>9271</v>
+        <v>9292</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>352</v>
       </c>
       <c r="B19">
-        <v>9198</v>
+        <v>9238</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8331</v>
+        <v>8377</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7445</v>
+        <v>7452</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>497</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>6933</v>
+        <v>7062</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260501_054421
📊 Data sync summary:
- Updated at: 2026-05-01 05:44:22 UTC
- Territories: 250
- IP ranges: 273648
- Data size: 43.65MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-04-30T05:30:19.549Z</t>
+    <t>2026-05-01T05:41:35.324Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 274896</t>
+    <t>Total IP ranges: 273648</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>274896</v>
+        <v>273648</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>289</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1902</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7452</v>
+        <v>7537</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2359</v>
+        <v>2382</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2123</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5263</v>
+        <v>4963</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5152</v>
+        <v>5226</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4613,7 +4613,7 @@
         <v>44</v>
       </c>
       <c r="I32">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1436</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>384</v>
+        <v>392</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9703</v>
+        <v>9525</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4903,7 +4903,7 @@
         <v>44</v>
       </c>
       <c r="I42">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1081</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4437</v>
+        <v>4455</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5106,7 +5106,7 @@
         <v>44</v>
       </c>
       <c r="I49">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1143</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>417</v>
+        <v>410</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1958</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1685</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>446</v>
+        <v>435</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>473</v>
+        <v>466</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>702</v>
+        <v>727</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>1942</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9238</v>
+        <v>9448</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16444</v>
+        <v>16371</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>749</v>
+        <v>732</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6527,7 +6527,7 @@
         <v>44</v>
       </c>
       <c r="I98">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7062</v>
+        <v>7310</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>964</v>
+        <v>970</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8377</v>
+        <v>8194</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4729</v>
+        <v>4750</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1630</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>396</v>
+        <v>401</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2276</v>
+        <v>2248</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1390</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5184</v>
+        <v>5247</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>6926</v>
+        <v>7353</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>991</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>524</v>
+        <v>533</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>725</v>
+        <v>733</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>893</v>
+        <v>965</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>582</v>
+        <v>590</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1571</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>190</v>
+        <v>146</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1867</v>
+        <v>1911</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>499</v>
+        <v>491</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12203</v>
+        <v>11786</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1560</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>536</v>
+        <v>564</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1761</v>
+        <v>1737</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>921</v>
+        <v>931</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>673</v>
+        <v>667</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1503</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5127</v>
+        <v>5194</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>774</v>
+        <v>775</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2430</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9292</v>
+        <v>9318</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9108,7 +9108,7 @@
         <v>44</v>
       </c>
       <c r="I187">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>982</v>
+        <v>970</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>362</v>
+        <v>369</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5695</v>
+        <v>5749</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9514,7 +9514,7 @@
         <v>44</v>
       </c>
       <c r="I201">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>594</v>
+        <v>588</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>610</v>
+        <v>614</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2400</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9688,7 +9688,7 @@
         <v>44</v>
       </c>
       <c r="I207">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2338</v>
+        <v>2377</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5521</v>
+        <v>5467</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3676</v>
+        <v>3604</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3530</v>
+        <v>3524</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1525</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>239</v>
+        <v>251</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1427</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2518</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3653</v>
+        <v>3628</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1201</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16719</v>
+        <v>16504</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>45256</v>
+        <v>43601</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10587,7 +10587,7 @@
         <v>44</v>
       </c>
       <c r="I238">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1411</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10819,7 +10819,7 @@
         <v>44</v>
       </c>
       <c r="I246">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="247" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>45256</v>
+        <v>43601</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>16719</v>
+        <v>16504</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>16444</v>
+        <v>16371</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12203</v>
+        <v>11786</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,23 +11143,23 @@
         <v>201</v>
       </c>
       <c r="B17">
-        <v>9703</v>
+        <v>9525</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B18">
-        <v>9292</v>
+        <v>9448</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>352</v>
+        <v>777</v>
       </c>
       <c r="B19">
-        <v>9238</v>
+        <v>9318</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8377</v>
+        <v>8194</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7452</v>
+        <v>7537</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>497</v>
       </c>
       <c r="B22">
-        <v>7062</v>
+        <v>7353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260515_055722
📊 Data sync summary:
- Updated at: 2026-05-15 05:57:23 UTC
- Territories: 250
- IP ranges: 274081
- Data size: 43.71MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-05-14T05:47:47.580Z</t>
+    <t>2026-05-15T05:54:40.781Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 273648</t>
+    <t>Total IP ranges: 274081</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>273648</v>
+        <v>274081</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>302</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1925</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7537</v>
+        <v>7419</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2382</v>
+        <v>2409</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2135</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4963</v>
+        <v>5644</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5226</v>
+        <v>5281</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1440</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9525</v>
+        <v>8741</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1102</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4455</v>
+        <v>4445</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5106,7 +5106,7 @@
         <v>44</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1152</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>410</v>
+        <v>429</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>405</v>
+        <v>395</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1970</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1698</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>435</v>
+        <v>439</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>2058</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9448</v>
+        <v>9439</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>344</v>
+        <v>354</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16371</v>
+        <v>16507</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>732</v>
+        <v>747</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7310</v>
+        <v>6871</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>970</v>
+        <v>964</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8194</v>
+        <v>8256</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4750</v>
+        <v>4805</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1629</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2248</v>
+        <v>2255</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1359</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5247</v>
+        <v>5259</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7353</v>
+        <v>7028</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1003</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>533</v>
+        <v>551</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>733</v>
+        <v>737</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>965</v>
+        <v>996</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>590</v>
+        <v>583</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1602</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1911</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11786</v>
+        <v>11728</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1559</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>564</v>
+        <v>552</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>931</v>
+        <v>924</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>299</v>
+        <v>309</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>667</v>
+        <v>783</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1521</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5194</v>
+        <v>5203</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>775</v>
+        <v>862</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>375</v>
+        <v>370</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>182</v>
+        <v>197</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2432</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9318</v>
+        <v>9360</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9224,7 +9224,7 @@
         <v>44</v>
       </c>
       <c r="I191">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>970</v>
+        <v>992</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>611</v>
+        <v>604</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5749</v>
+        <v>5868</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>614</v>
+        <v>615</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2504</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2377</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5467</v>
+        <v>5668</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3604</v>
+        <v>3599</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3524</v>
+        <v>3568</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1541</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1467</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2563</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3628</v>
+        <v>3653</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1194</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16504</v>
+        <v>16646</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43601</v>
+        <v>43523</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>325</v>
+        <v>333</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>492</v>
+        <v>507</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1423</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43601</v>
+        <v>43523</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>16504</v>
+        <v>16646</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>16371</v>
+        <v>16507</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,31 +11135,31 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11786</v>
+        <v>11728</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>201</v>
+        <v>352</v>
       </c>
       <c r="B17">
-        <v>9525</v>
+        <v>9439</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>352</v>
+        <v>777</v>
       </c>
       <c r="B18">
-        <v>9448</v>
+        <v>9360</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>777</v>
+        <v>201</v>
       </c>
       <c r="B19">
-        <v>9318</v>
+        <v>8741</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8194</v>
+        <v>8256</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7537</v>
+        <v>7419</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>497</v>
       </c>
       <c r="B22">
-        <v>7353</v>
+        <v>7028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260601_065803
📊 Data sync summary:
- Updated at: 2026-06-01 06:58:04 UTC
- Territories: 250
- IP ranges: 274987
- Data size: 43.86MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-05-31T06:18:28.006Z</t>
+    <t>2026-06-01T06:55:24.557Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 274081</t>
+    <t>Total IP ranges: 274987</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>274081</v>
+        <v>274987</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>310</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>51</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>2074</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>216</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7419</v>
+        <v>7487</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2409</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>232</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2145</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>5644</v>
+        <v>4156</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>151</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5281</v>
+        <v>5309</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1425</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>25</v>
       </c>
       <c r="I37">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>388</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>8741</v>
+        <v>9717</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1078</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4445</v>
+        <v>4447</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1159</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>395</v>
+        <v>399</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1985</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1684</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>463</v>
+        <v>480</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>726</v>
+        <v>724</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>2050</v>
+        <v>2083</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9439</v>
+        <v>9514</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>354</v>
+        <v>364</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16507</v>
+        <v>16713</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6871</v>
+        <v>7145</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>964</v>
+        <v>951</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8256</v>
+        <v>8129</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4805</v>
+        <v>4792</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1632</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2255</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1379</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5259</v>
+        <v>5181</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7028</v>
+        <v>7122</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1013</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>551</v>
+        <v>569</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>192</v>
+        <v>205</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>171</v>
+        <v>183</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>737</v>
+        <v>734</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>996</v>
+        <v>961</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>583</v>
+        <v>594</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1615</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>142</v>
+        <v>194</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1931</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>490</v>
+        <v>494</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>307</v>
+        <v>314</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>298</v>
+        <v>305</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>11728</v>
+        <v>12069</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1562</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>552</v>
+        <v>547</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1737</v>
+        <v>1717</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>924</v>
+        <v>933</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>783</v>
+        <v>798</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1506</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5203</v>
+        <v>5291</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>862</v>
+        <v>827</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>197</v>
+        <v>180</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2447</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9360</v>
+        <v>9511</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>992</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>367</v>
+        <v>318</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5868</v>
+        <v>5969</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>615</v>
+        <v>611</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2513</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2433</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5668</v>
+        <v>5530</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3599</v>
+        <v>3711</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3568</v>
+        <v>3535</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -10007,7 +10007,7 @@
         <v>25</v>
       </c>
       <c r="I218">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1521</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>252</v>
+        <v>265</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1471</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2619</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3653</v>
+        <v>3610</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1205</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16646</v>
+        <v>16625</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43523</v>
+        <v>43679</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>507</v>
+        <v>492</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1422</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,23 +11111,23 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43523</v>
+        <v>43679</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>989</v>
+        <v>380</v>
       </c>
       <c r="B14">
-        <v>16646</v>
+        <v>16713</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>380</v>
+        <v>989</v>
       </c>
       <c r="B15">
-        <v>16507</v>
+        <v>16625</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,31 +11135,31 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>11728</v>
+        <v>12069</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>352</v>
+        <v>201</v>
       </c>
       <c r="B17">
-        <v>9439</v>
+        <v>9717</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>777</v>
+        <v>352</v>
       </c>
       <c r="B18">
-        <v>9360</v>
+        <v>9514</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>201</v>
+        <v>777</v>
       </c>
       <c r="B19">
-        <v>8741</v>
+        <v>9511</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8256</v>
+        <v>8129</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7419</v>
+        <v>7487</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>497</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>7028</v>
+        <v>7145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260615_072305
📊 Data sync summary:
- Updated at: 2026-06-15 07:23:07 UTC
- Territories: 250
- IP ranges: 276451
- Data size: 44.09MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-06-14T06:40:08.945Z</t>
+    <t>2026-06-15T07:20:20.567Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 274987</t>
+    <t>Total IP ranges: 276451</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>274987</v>
+        <v>276451</v>
       </c>
     </row>
   </sheetData>
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3830,7 +3830,7 @@
         <v>44</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>2086</v>
+        <v>2107</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7487</v>
+        <v>7503</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2447</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2120</v>
+        <v>2121</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4156</v>
+        <v>4351</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5309</v>
+        <v>5388</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1462</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9717</v>
+        <v>9638</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1075</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4447</v>
+        <v>4442</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1175</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>431</v>
+        <v>444</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>399</v>
+        <v>426</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1995</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1719</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>437</v>
+        <v>446</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>317</v>
+        <v>339</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>724</v>
+        <v>751</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5831,7 +5831,7 @@
         <v>44</v>
       </c>
       <c r="I74">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>2083</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9514</v>
+        <v>9623</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16713</v>
+        <v>16738</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>746</v>
+        <v>747</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7145</v>
+        <v>7108</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>951</v>
+        <v>960</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8129</v>
+        <v>8217</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4792</v>
+        <v>4811</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1633</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2188</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1407</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5181</v>
+        <v>5198</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7122</v>
+        <v>7166</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>180</v>
+        <v>192</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1015</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>205</v>
+        <v>194</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>961</v>
+        <v>944</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>594</v>
+        <v>615</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1632</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7687,7 +7687,7 @@
         <v>25</v>
       </c>
       <c r="I138">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1935</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>494</v>
+        <v>498</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>314</v>
+        <v>307</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12069</v>
+        <v>12190</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1565</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1717</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>933</v>
+        <v>944</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>305</v>
+        <v>351</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>798</v>
+        <v>795</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1546</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5291</v>
+        <v>5316</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2460</v>
+        <v>2485</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9511</v>
+        <v>9421</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9224,7 +9224,7 @@
         <v>44</v>
       </c>
       <c r="I191">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>1006</v>
+        <v>988</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>606</v>
+        <v>618</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>318</v>
+        <v>309</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5969</v>
+        <v>6194</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2430</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2432</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5530</v>
+        <v>5562</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3711</v>
+        <v>3704</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3535</v>
+        <v>3559</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1525</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1463</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2598</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3610</v>
+        <v>3522</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1165</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16625</v>
+        <v>16865</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43679</v>
+        <v>43842</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>492</v>
+        <v>497</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1452</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,23 +11111,23 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43679</v>
+        <v>43842</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>380</v>
+        <v>989</v>
       </c>
       <c r="B14">
-        <v>16713</v>
+        <v>16865</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>989</v>
+        <v>380</v>
       </c>
       <c r="B15">
-        <v>16625</v>
+        <v>16738</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12069</v>
+        <v>12190</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>201</v>
       </c>
       <c r="B17">
-        <v>9717</v>
+        <v>9638</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>9514</v>
+        <v>9623</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>777</v>
       </c>
       <c r="B19">
-        <v>9511</v>
+        <v>9421</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8129</v>
+        <v>8217</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7487</v>
+        <v>7503</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>497</v>
       </c>
       <c r="B22">
-        <v>7145</v>
+        <v>7166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260701_062858
📊 Data sync summary:
- Updated at: 2026-07-01 06:28:59 UTC
- Territories: 250
- IP ranges: 283445
- Data size: 45.20MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-06-30T06:11:35.526Z</t>
+    <t>2026-07-01T06:26:21.018Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 276451</t>
+    <t>Total IP ranges: 283445</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>276451</v>
+        <v>283445</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>2107</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7503</v>
+        <v>7560</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2496</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2121</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>4351</v>
+        <v>6541</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5388</v>
+        <v>5451</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1473</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9638</v>
+        <v>11109</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1079</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4442</v>
+        <v>4436</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1177</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>356</v>
+        <v>350</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>444</v>
+        <v>433</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>426</v>
+        <v>409</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>2019</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>1701</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>446</v>
+        <v>442</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>339</v>
+        <v>311</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>751</v>
+        <v>720</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5831,7 +5831,7 @@
         <v>44</v>
       </c>
       <c r="I74">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>2120</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9623</v>
+        <v>9862</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>367</v>
+        <v>354</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16738</v>
+        <v>16890</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>747</v>
+        <v>723</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>25</v>
       </c>
       <c r="I94">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7108</v>
+        <v>7229</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>960</v>
+        <v>910</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>223</v>
+        <v>214</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8217</v>
+        <v>8070</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4811</v>
+        <v>4840</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1643</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2197</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1368</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5198</v>
+        <v>5245</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7166</v>
+        <v>7109</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>194</v>
+        <v>202</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>733</v>
+        <v>772</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>944</v>
+        <v>954</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>615</v>
+        <v>605</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7803,7 +7803,7 @@
         <v>44</v>
       </c>
       <c r="I142">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>1948</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>498</v>
+        <v>534</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>44</v>
       </c>
       <c r="I149">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>140</v>
+        <v>163</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12190</v>
+        <v>12271</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1573</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>549</v>
+        <v>543</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1716</v>
+        <v>1757</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>944</v>
+        <v>936</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>351</v>
+        <v>291</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>795</v>
+        <v>661</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1558</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5316</v>
+        <v>5231</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>826</v>
+        <v>832</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2485</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9224,7 +9224,7 @@
         <v>44</v>
       </c>
       <c r="I191">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>988</v>
+        <v>989</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>618</v>
+        <v>613</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>309</v>
+        <v>325</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>6194</v>
+        <v>6392</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>590</v>
+        <v>596</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>611</v>
+        <v>603</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2378</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2451</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5562</v>
+        <v>5592</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3704</v>
+        <v>3758</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3559</v>
+        <v>3697</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1549</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>264</v>
+        <v>253</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1474</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10384,7 +10384,7 @@
         <v>25</v>
       </c>
       <c r="I231">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2591</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3522</v>
+        <v>3545</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1151</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>16865</v>
+        <v>17092</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>43842</v>
+        <v>46055</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>336</v>
+        <v>340</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>497</v>
+        <v>502</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1439</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>43842</v>
+        <v>46055</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>16865</v>
+        <v>17092</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>16738</v>
+        <v>16890</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12190</v>
+        <v>12271</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>201</v>
       </c>
       <c r="B17">
-        <v>9638</v>
+        <v>11109</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>9623</v>
+        <v>9862</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8217</v>
+        <v>8070</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7503</v>
+        <v>7560</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>497</v>
+        <v>445</v>
       </c>
       <c r="B22">
-        <v>7166</v>
+        <v>7229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260715_045428
📊 Data sync summary:
- Updated at: 2026-07-15 04:54:29 UTC
- Territories: 250
- IP ranges: 283818
- Data size: 45.26MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-07-14T04:50:48.486Z</t>
+    <t>2026-07-15T04:51:40.134Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 283445</t>
+    <t>Total IP ranges: 283818</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>283445</v>
+        <v>283818</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>300</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1940</v>
+        <v>2102</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>233</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7560</v>
+        <v>7532</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2489</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2135</v>
+        <v>2132</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>6541</v>
+        <v>6594</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5451</v>
+        <v>5455</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1455</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>11109</v>
+        <v>9944</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1090</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4436</v>
+        <v>4472</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1178</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>409</v>
+        <v>416</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1994</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>2048</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>442</v>
+        <v>445</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>480</v>
+        <v>474</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>311</v>
+        <v>334</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>720</v>
+        <v>739</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>44</v>
       </c>
       <c r="I73">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -5831,7 +5831,7 @@
         <v>44</v>
       </c>
       <c r="I74">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>2126</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9862</v>
+        <v>9845</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>354</v>
+        <v>370</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16890</v>
+        <v>16853</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>723</v>
+        <v>742</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7229</v>
+        <v>7014</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>910</v>
+        <v>930</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8070</v>
+        <v>8186</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4840</v>
+        <v>4875</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1648</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2188</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1354</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5245</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7109</v>
+        <v>7183</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1021</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>567</v>
+        <v>587</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>772</v>
+        <v>779</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>111</v>
+        <v>130</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>954</v>
+        <v>951</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>605</v>
+        <v>589</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7513,7 +7513,7 @@
         <v>25</v>
       </c>
       <c r="I132">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1623</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>2009</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12271</v>
+        <v>12348</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1554</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>543</v>
+        <v>552</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1757</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>936</v>
+        <v>945</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8615,7 +8615,7 @@
         <v>25</v>
       </c>
       <c r="I170">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>661</v>
+        <v>767</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1523</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5231</v>
+        <v>5280</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>832</v>
+        <v>839</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2454</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9421</v>
+        <v>9460</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>989</v>
+        <v>998</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>613</v>
+        <v>616</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>6392</v>
+        <v>5920</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>596</v>
+        <v>615</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>603</v>
+        <v>606</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2439</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2463</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5592</v>
+        <v>5613</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3758</v>
+        <v>3819</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3697</v>
+        <v>3723</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1575</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1486</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10181,7 +10181,7 @@
         <v>25</v>
       </c>
       <c r="I224">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2539</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3545</v>
+        <v>3547</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1196</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>17092</v>
+        <v>17645</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>46055</v>
+        <v>46056</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>502</v>
+        <v>515</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1448</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>46055</v>
+        <v>46056</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>17092</v>
+        <v>17645</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>16890</v>
+        <v>16853</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12271</v>
+        <v>12348</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>201</v>
       </c>
       <c r="B17">
-        <v>11109</v>
+        <v>9944</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>352</v>
       </c>
       <c r="B18">
-        <v>9862</v>
+        <v>9845</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>777</v>
       </c>
       <c r="B19">
-        <v>9421</v>
+        <v>9460</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8070</v>
+        <v>8186</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,15 +11175,15 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7560</v>
+        <v>7532</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>497</v>
       </c>
       <c r="B22">
-        <v>7229</v>
+        <v>7183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260801_052926
📊 Data sync summary:
- Updated at: 2026-08-01 05:29:27 UTC
- Territories: 250
- IP ranges: 286753
- Data size: 45.73MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-07-31T05:35:46.905Z</t>
+    <t>2026-08-01T05:26:50.432Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 283818</t>
+    <t>Total IP ranges: 286753</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>283818</v>
+        <v>286753</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>2102</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7532</v>
+        <v>7487</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2490</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2132</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>6594</v>
+        <v>6520</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5455</v>
+        <v>5577</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>139</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1474</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>381</v>
+        <v>373</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4816,7 +4816,7 @@
         <v>25</v>
       </c>
       <c r="I39">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9944</v>
+        <v>9942</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
         <v>25</v>
       </c>
       <c r="I41">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1082</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4472</v>
+        <v>4480</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1196</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>44</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>416</v>
+        <v>403</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>2043</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>2043</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>445</v>
+        <v>461</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>334</v>
+        <v>309</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>739</v>
+        <v>752</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>2135</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>9845</v>
+        <v>10556</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>370</v>
+        <v>377</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>16853</v>
+        <v>17090</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>742</v>
+        <v>729</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6324,7 +6324,7 @@
         <v>44</v>
       </c>
       <c r="I91">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
@@ -6382,7 +6382,7 @@
         <v>44</v>
       </c>
       <c r="I93">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>232</v>
+        <v>240</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>7014</v>
+        <v>6783</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>930</v>
+        <v>918</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8186</v>
+        <v>8280</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4875</v>
+        <v>4866</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1653</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2236</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1385</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5307</v>
+        <v>5876</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7183</v>
+        <v>7109</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1026</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>779</v>
+        <v>774</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>130</v>
+        <v>106</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>951</v>
+        <v>960</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1664</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>2027</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>523</v>
+        <v>546</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12348</v>
+        <v>12119</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>552</v>
+        <v>548</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1758</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>945</v>
+        <v>947</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>288</v>
+        <v>280</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>767</v>
+        <v>792</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1563</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8818,7 +8818,7 @@
         <v>44</v>
       </c>
       <c r="I177">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5280</v>
+        <v>5285</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>839</v>
+        <v>776</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>377</v>
+        <v>372</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2495</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9460</v>
+        <v>9478</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>998</v>
+        <v>995</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>616</v>
+        <v>624</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>319</v>
+        <v>307</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5920</v>
+        <v>5671</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>615</v>
+        <v>586</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2464</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2555</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5613</v>
+        <v>5617</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3819</v>
+        <v>3780</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3723</v>
+        <v>3725</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1570</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1503</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2605</v>
+        <v>2618</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3547</v>
+        <v>3564</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1229</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>17645</v>
+        <v>18665</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>46056</v>
+        <v>46898</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>338</v>
+        <v>344</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>515</v>
+        <v>530</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1458</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>25</v>
       </c>
       <c r="I248">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -10964,7 +10964,7 @@
         <v>44</v>
       </c>
       <c r="I251">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>46056</v>
+        <v>46898</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>17645</v>
+        <v>18665</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>16853</v>
+        <v>17090</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,23 +11135,23 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12348</v>
+        <v>12119</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>201</v>
+        <v>352</v>
       </c>
       <c r="B17">
-        <v>9944</v>
+        <v>10556</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>352</v>
+        <v>201</v>
       </c>
       <c r="B18">
-        <v>9845</v>
+        <v>9942</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>777</v>
       </c>
       <c r="B19">
-        <v>9460</v>
+        <v>9478</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8186</v>
+        <v>8280</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7532</v>
+        <v>7487</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>497</v>
       </c>
       <c r="B22">
-        <v>7183</v>
+        <v>7109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260815_025346
📊 Data sync summary:
- Updated at: 2026-08-15 02:53:48 UTC
- Territories: 250
- IP ranges: 286137
- Data size: 45.63MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-08-14T04:07:46.118Z</t>
+    <t>2026-08-15T02:51:02.319Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 286753</t>
+    <t>Total IP ranges: 286137</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>286753</v>
+        <v>286137</v>
       </c>
     </row>
   </sheetData>
@@ -3743,7 +3743,7 @@
         <v>25</v>
       </c>
       <c r="I2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>25</v>
       </c>
       <c r="I3">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -3801,7 +3801,7 @@
         <v>25</v>
       </c>
       <c r="I4">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3888,7 +3888,7 @@
         <v>25</v>
       </c>
       <c r="I7">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>2091</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7487</v>
+        <v>7540</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2471</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>251</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2140</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>25</v>
       </c>
       <c r="I20">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>221</v>
+        <v>235</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>6520</v>
+        <v>6332</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>25</v>
       </c>
       <c r="I24">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4526,7 +4526,7 @@
         <v>25</v>
       </c>
       <c r="I29">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5577</v>
+        <v>5593</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4729,7 +4729,7 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9942</v>
+        <v>9166</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4961,7 +4961,7 @@
         <v>25</v>
       </c>
       <c r="I44">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -4990,7 +4990,7 @@
         <v>25</v>
       </c>
       <c r="I45">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1102</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4480</v>
+        <v>4477</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1197</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>25</v>
       </c>
       <c r="I51">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>25</v>
       </c>
       <c r="I52">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>403</v>
+        <v>409</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>2007</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5425,7 +5425,7 @@
         <v>25</v>
       </c>
       <c r="I60">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>2040</v>
+        <v>2082</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>23</v>
+        <v>33</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>461</v>
+        <v>454</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>471</v>
+        <v>485</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>309</v>
+        <v>329</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>752</v>
+        <v>773</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="I71">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -5773,7 +5773,7 @@
         <v>25</v>
       </c>
       <c r="I72">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>25</v>
       </c>
       <c r="I75">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>10556</v>
+        <v>10704</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -5976,7 +5976,7 @@
         <v>44</v>
       </c>
       <c r="I79">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6063,7 +6063,7 @@
         <v>25</v>
       </c>
       <c r="I82">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>17090</v>
+        <v>17040</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>196</v>
+        <v>216</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>729</v>
+        <v>744</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6353,7 +6353,7 @@
         <v>25</v>
       </c>
       <c r="I92">
-        <v>255</v>
+        <v>284</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
@@ -6440,7 +6440,7 @@
         <v>25</v>
       </c>
       <c r="I95">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6783</v>
+        <v>6912</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>918</v>
+        <v>911</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>218</v>
+        <v>225</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8280</v>
+        <v>8335</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4866</v>
+        <v>4915</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1752</v>
+        <v>1770</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>403</v>
+        <v>409</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2306</v>
+        <v>2258</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1487</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5876</v>
+        <v>5894</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6933,7 +6933,7 @@
         <v>25</v>
       </c>
       <c r="I112">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7109</v>
+        <v>7177</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1033</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>589</v>
+        <v>606</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7165,7 +7165,7 @@
         <v>25</v>
       </c>
       <c r="I120">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>774</v>
+        <v>785</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>25</v>
       </c>
       <c r="I125">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
@@ -7339,7 +7339,7 @@
         <v>25</v>
       </c>
       <c r="I126">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>960</v>
+        <v>945</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1643</v>
+        <v>1697</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7745,7 @@
         <v>25</v>
       </c>
       <c r="I140">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>188</v>
+        <v>444</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>2005</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7861,7 +7861,7 @@
         <v>25</v>
       </c>
       <c r="I144">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>546</v>
+        <v>530</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -7977,7 +7977,7 @@
         <v>25</v>
       </c>
       <c r="I148">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>155</v>
+        <v>162</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>322</v>
+        <v>317</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8122,7 +8122,7 @@
         <v>25</v>
       </c>
       <c r="I153">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>25</v>
       </c>
       <c r="I154">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12119</v>
+        <v>12271</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1570</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>548</v>
+        <v>574</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8383,7 +8383,7 @@
         <v>44</v>
       </c>
       <c r="I162">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1738</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>947</v>
+        <v>967</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>280</v>
+        <v>291</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>245</v>
+        <v>254</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>792</v>
+        <v>700</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1562</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5285</v>
+        <v>5328</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>776</v>
+        <v>759</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>372</v>
+        <v>378</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>190</v>
+        <v>181</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2545</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9050,7 +9050,7 @@
         <v>44</v>
       </c>
       <c r="I185">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -9137,7 +9137,7 @@
         <v>25</v>
       </c>
       <c r="I188">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -9166,7 +9166,7 @@
         <v>25</v>
       </c>
       <c r="I189">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -9195,7 +9195,7 @@
         <v>44</v>
       </c>
       <c r="I190">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>995</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>624</v>
+        <v>625</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>307</v>
+        <v>320</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5671</v>
+        <v>5795</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>586</v>
+        <v>594</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>613</v>
+        <v>624</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9630,7 +9630,7 @@
         <v>25</v>
       </c>
       <c r="I205">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2465</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2531</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5617</v>
+        <v>5614</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>25</v>
       </c>
       <c r="I213">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>25</v>
       </c>
       <c r="I215">
-        <v>3780</v>
+        <v>3881</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3725</v>
+        <v>3760</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1575</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>256</v>
+        <v>264</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1509</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10152,7 +10152,7 @@
         <v>25</v>
       </c>
       <c r="I223">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10297,7 +10297,7 @@
         <v>25</v>
       </c>
       <c r="I228">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10355,7 +10355,7 @@
         <v>44</v>
       </c>
       <c r="I230">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2618</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10442,7 +10442,7 @@
         <v>25</v>
       </c>
       <c r="I233">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3564</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1252</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>18665</v>
+        <v>18360</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>46898</v>
+        <v>46016</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>530</v>
+        <v>526</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1459</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -10935,7 +10935,7 @@
         <v>25</v>
       </c>
       <c r="I250">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>46898</v>
+        <v>46016</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>18665</v>
+        <v>18360</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>17090</v>
+        <v>17040</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12119</v>
+        <v>12271</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,23 +11143,23 @@
         <v>352</v>
       </c>
       <c r="B17">
-        <v>10556</v>
+        <v>10704</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>777</v>
       </c>
       <c r="B18">
-        <v>9942</v>
+        <v>9478</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>777</v>
+        <v>201</v>
       </c>
       <c r="B19">
-        <v>9478</v>
+        <v>9166</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8280</v>
+        <v>8335</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7487</v>
+        <v>7540</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>497</v>
       </c>
       <c r="B22">
-        <v>7109</v>
+        <v>7177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update geo-ip data - 20260901_071957
📊 Data sync summary:
- Updated at: 2026-09-01 07:19:59 UTC
- Territories: 250
- IP ranges: 284973
- Data size: 45.44MB

🤖 Auto-generated by GitHub Actions
</commit_message>
<xml_diff>
--- a/data/combined-geo-ip-data.xlsx
+++ b/data/combined-geo-ip-data.xlsx
@@ -22,7 +22,7 @@
     <t>Generated at:</t>
   </si>
   <si>
-    <t>2026-08-31T08:07:55.124Z</t>
+    <t>2026-09-01T07:17:13.118Z</t>
   </si>
   <si>
     <t>Metric</t>
@@ -3172,7 +3172,7 @@
     <t>IP Ranges Data Too Large</t>
   </si>
   <si>
-    <t>Total IP ranges: 286137</t>
+    <t>Total IP ranges: 284973</t>
   </si>
   <si>
     <t>The IP ranges data is too large to include in Excel format.</t>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>286137</v>
+        <v>284973</v>
       </c>
     </row>
   </sheetData>
@@ -3859,7 +3859,7 @@
         <v>25</v>
       </c>
       <c r="I6">
-        <v>67</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3946,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="I9">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3975,7 +3975,7 @@
         <v>25</v>
       </c>
       <c r="I10">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -4004,7 +4004,7 @@
         <v>25</v>
       </c>
       <c r="I11">
-        <v>1972</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="I12">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>25</v>
       </c>
       <c r="I14">
-        <v>7540</v>
+        <v>7554</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -4120,7 +4120,7 @@
         <v>25</v>
       </c>
       <c r="I15">
-        <v>2474</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -4149,7 +4149,7 @@
         <v>25</v>
       </c>
       <c r="I16">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="I17">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4207,7 +4207,7 @@
         <v>25</v>
       </c>
       <c r="I18">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4236,7 +4236,7 @@
         <v>25</v>
       </c>
       <c r="I19">
-        <v>2163</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4294,7 +4294,7 @@
         <v>25</v>
       </c>
       <c r="I21">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="I22">
-        <v>6332</v>
+        <v>6225</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4352,7 +4352,7 @@
         <v>25</v>
       </c>
       <c r="I23">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4410,7 +4410,7 @@
         <v>44</v>
       </c>
       <c r="I25">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -4439,7 +4439,7 @@
         <v>25</v>
       </c>
       <c r="I26">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>25</v>
       </c>
       <c r="I27">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -4497,7 +4497,7 @@
         <v>25</v>
       </c>
       <c r="I28">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -4555,7 +4555,7 @@
         <v>44</v>
       </c>
       <c r="I30">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4584,7 +4584,7 @@
         <v>25</v>
       </c>
       <c r="I31">
-        <v>5593</v>
+        <v>5493</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>44</v>
       </c>
       <c r="I33">
-        <v>131</v>
+        <v>143</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>25</v>
       </c>
       <c r="I34">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4700,7 +4700,7 @@
         <v>25</v>
       </c>
       <c r="I35">
-        <v>1486</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>25</v>
       </c>
       <c r="I38">
-        <v>376</v>
+        <v>383</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -4845,7 +4845,7 @@
         <v>25</v>
       </c>
       <c r="I40">
-        <v>9166</v>
+        <v>9270</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -4932,7 +4932,7 @@
         <v>44</v>
       </c>
       <c r="I43">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -5019,7 +5019,7 @@
         <v>25</v>
       </c>
       <c r="I46">
-        <v>1108</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>25</v>
       </c>
       <c r="I47">
-        <v>4477</v>
+        <v>4501</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>25</v>
       </c>
       <c r="I50">
-        <v>1194</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>25</v>
       </c>
       <c r="I54">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="I55">
-        <v>437</v>
+        <v>424</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -5309,7 +5309,7 @@
         <v>25</v>
       </c>
       <c r="I56">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5338,7 +5338,7 @@
         <v>44</v>
       </c>
       <c r="I57">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>25</v>
       </c>
       <c r="I58">
-        <v>409</v>
+        <v>403</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -5396,7 +5396,7 @@
         <v>25</v>
       </c>
       <c r="I59">
-        <v>1997</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -5454,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="I61">
-        <v>2082</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -5483,7 +5483,7 @@
         <v>25</v>
       </c>
       <c r="I62">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -5512,7 +5512,7 @@
         <v>25</v>
       </c>
       <c r="I63">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -5541,7 +5541,7 @@
         <v>25</v>
       </c>
       <c r="I64">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>25</v>
       </c>
       <c r="I65">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -5599,7 +5599,7 @@
         <v>25</v>
       </c>
       <c r="I66">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -5628,7 +5628,7 @@
         <v>25</v>
       </c>
       <c r="I67">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -5657,7 +5657,7 @@
         <v>25</v>
       </c>
       <c r="I68">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -5686,7 +5686,7 @@
         <v>25</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
@@ -5715,7 +5715,7 @@
         <v>25</v>
       </c>
       <c r="I70">
-        <v>773</v>
+        <v>769</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>25</v>
       </c>
       <c r="I76">
-        <v>2153</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>25</v>
       </c>
       <c r="I77">
-        <v>10704</v>
+        <v>9982</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>44</v>
       </c>
       <c r="I78">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="I81">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
@@ -6092,7 +6092,7 @@
         <v>25</v>
       </c>
       <c r="I83">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
@@ -6121,7 +6121,7 @@
         <v>25</v>
       </c>
       <c r="I84">
-        <v>17040</v>
+        <v>17086</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,7 +6150,7 @@
         <v>25</v>
       </c>
       <c r="I85">
-        <v>216</v>
+        <v>210</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
@@ -6179,7 +6179,7 @@
         <v>44</v>
       </c>
       <c r="I86">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
@@ -6208,7 +6208,7 @@
         <v>25</v>
       </c>
       <c r="I87">
-        <v>744</v>
+        <v>760</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>44</v>
       </c>
       <c r="I88">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
@@ -6266,7 +6266,7 @@
         <v>25</v>
       </c>
       <c r="I89">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -6295,7 +6295,7 @@
         <v>44</v>
       </c>
       <c r="I90">
-        <v>93</v>
+        <v>71</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -6469,7 +6469,7 @@
         <v>25</v>
       </c>
       <c r="I96">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>25</v>
       </c>
       <c r="I97">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
@@ -6556,7 +6556,7 @@
         <v>25</v>
       </c>
       <c r="I99">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -6585,7 +6585,7 @@
         <v>44</v>
       </c>
       <c r="I100">
-        <v>6912</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -6614,7 +6614,7 @@
         <v>25</v>
       </c>
       <c r="I101">
-        <v>911</v>
+        <v>931</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>25</v>
       </c>
       <c r="I102">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -6672,7 +6672,7 @@
         <v>25</v>
       </c>
       <c r="I103">
-        <v>8335</v>
+        <v>8250</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -6701,7 +6701,7 @@
         <v>25</v>
       </c>
       <c r="I104">
-        <v>4915</v>
+        <v>4950</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>25</v>
       </c>
       <c r="I105">
-        <v>1770</v>
+        <v>1773</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
@@ -6759,7 +6759,7 @@
         <v>25</v>
       </c>
       <c r="I106">
-        <v>409</v>
+        <v>403</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
@@ -6788,7 +6788,7 @@
         <v>25</v>
       </c>
       <c r="I107">
-        <v>2258</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>44</v>
       </c>
       <c r="I108">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
@@ -6846,7 +6846,7 @@
         <v>25</v>
       </c>
       <c r="I109">
-        <v>1500</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
         <v>25</v>
       </c>
       <c r="I110">
-        <v>5894</v>
+        <v>5402</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -6904,7 +6904,7 @@
         <v>25</v>
       </c>
       <c r="I111">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
@@ -6962,7 +6962,7 @@
         <v>25</v>
       </c>
       <c r="I113">
-        <v>7177</v>
+        <v>7336</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>44</v>
       </c>
       <c r="I114">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
@@ -7020,7 +7020,7 @@
         <v>25</v>
       </c>
       <c r="I115">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -7049,7 +7049,7 @@
         <v>25</v>
       </c>
       <c r="I116">
-        <v>1042</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
@@ -7078,7 +7078,7 @@
         <v>25</v>
       </c>
       <c r="I117">
-        <v>606</v>
+        <v>603</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
@@ -7107,7 +7107,7 @@
         <v>25</v>
       </c>
       <c r="I118">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
@@ -7194,7 +7194,7 @@
         <v>25</v>
       </c>
       <c r="I121">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>25</v>
       </c>
       <c r="I122">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
@@ -7252,7 +7252,7 @@
         <v>25</v>
       </c>
       <c r="I123">
-        <v>785</v>
+        <v>781</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>25</v>
       </c>
       <c r="I124">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
@@ -7368,7 +7368,7 @@
         <v>25</v>
       </c>
       <c r="I127">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>25</v>
       </c>
       <c r="I128">
-        <v>119</v>
+        <v>110</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
@@ -7426,7 +7426,7 @@
         <v>25</v>
       </c>
       <c r="I129">
-        <v>945</v>
+        <v>949</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
@@ -7455,7 +7455,7 @@
         <v>25</v>
       </c>
       <c r="I130">
-        <v>588</v>
+        <v>608</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -7484,7 +7484,7 @@
         <v>44</v>
       </c>
       <c r="I131">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
         <v>25</v>
       </c>
       <c r="I133">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>25</v>
       </c>
       <c r="I134">
-        <v>1697</v>
+        <v>1747</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>25</v>
       </c>
       <c r="I135">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
@@ -7629,7 +7629,7 @@
         <v>25</v>
       </c>
       <c r="I136">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
@@ -7658,7 +7658,7 @@
         <v>25</v>
       </c>
       <c r="I137">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
@@ -7716,7 +7716,7 @@
         <v>44</v>
       </c>
       <c r="I139">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
@@ -7774,7 +7774,7 @@
         <v>25</v>
       </c>
       <c r="I141">
-        <v>444</v>
+        <v>317</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>25</v>
       </c>
       <c r="I143">
-        <v>2048</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
@@ -7890,7 +7890,7 @@
         <v>25</v>
       </c>
       <c r="I145">
-        <v>530</v>
+        <v>512</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
@@ -7919,7 +7919,7 @@
         <v>25</v>
       </c>
       <c r="I146">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
         <v>25</v>
       </c>
       <c r="I147">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
@@ -8035,7 +8035,7 @@
         <v>25</v>
       </c>
       <c r="I150">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
@@ -8064,7 +8064,7 @@
         <v>25</v>
       </c>
       <c r="I151">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
@@ -8093,7 +8093,7 @@
         <v>25</v>
       </c>
       <c r="I152">
-        <v>317</v>
+        <v>328</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
         <v>25</v>
       </c>
       <c r="I155">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
@@ -8209,7 +8209,7 @@
         <v>25</v>
       </c>
       <c r="I156">
-        <v>12271</v>
+        <v>12264</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -8238,7 +8238,7 @@
         <v>44</v>
       </c>
       <c r="I157">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
@@ -8267,7 +8267,7 @@
         <v>25</v>
       </c>
       <c r="I158">
-        <v>1574</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -8296,7 +8296,7 @@
         <v>25</v>
       </c>
       <c r="I159">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
@@ -8325,7 +8325,7 @@
         <v>25</v>
       </c>
       <c r="I160">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
@@ -8354,7 +8354,7 @@
         <v>25</v>
       </c>
       <c r="I161">
-        <v>574</v>
+        <v>555</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
@@ -8470,7 +8470,7 @@
         <v>25</v>
       </c>
       <c r="I165">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
@@ -8499,7 +8499,7 @@
         <v>44</v>
       </c>
       <c r="I166">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
@@ -8528,7 +8528,7 @@
         <v>25</v>
       </c>
       <c r="I167">
-        <v>1851</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="I168">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>25</v>
       </c>
       <c r="I169">
-        <v>967</v>
+        <v>974</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
@@ -8644,7 +8644,7 @@
         <v>44</v>
       </c>
       <c r="I171">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
@@ -8673,7 +8673,7 @@
         <v>25</v>
       </c>
       <c r="I172">
-        <v>291</v>
+        <v>295</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
@@ -8702,7 +8702,7 @@
         <v>25</v>
       </c>
       <c r="I173">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="I174">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="I175">
-        <v>700</v>
+        <v>679</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
@@ -8789,7 +8789,7 @@
         <v>25</v>
       </c>
       <c r="I176">
-        <v>1561</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>25</v>
       </c>
       <c r="I178">
-        <v>5328</v>
+        <v>5377</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -8876,7 +8876,7 @@
         <v>25</v>
       </c>
       <c r="I179">
-        <v>759</v>
+        <v>775</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>44</v>
       </c>
       <c r="I180">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8934,7 +8934,7 @@
         <v>25</v>
       </c>
       <c r="I181">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8963,7 +8963,7 @@
         <v>25</v>
       </c>
       <c r="I182">
-        <v>2535</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8992,7 +8992,7 @@
         <v>25</v>
       </c>
       <c r="I183">
-        <v>9478</v>
+        <v>9492</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -9021,7 +9021,7 @@
         <v>25</v>
       </c>
       <c r="I184">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -9079,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="I186">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -9253,7 +9253,7 @@
         <v>25</v>
       </c>
       <c r="I192">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
@@ -9282,7 +9282,7 @@
         <v>25</v>
       </c>
       <c r="I193">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>25</v>
       </c>
       <c r="I194">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
@@ -9340,7 +9340,7 @@
         <v>25</v>
       </c>
       <c r="I195">
-        <v>1011</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>25</v>
       </c>
       <c r="I196">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
@@ -9398,7 +9398,7 @@
         <v>25</v>
       </c>
       <c r="I197">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
@@ -9427,7 +9427,7 @@
         <v>25</v>
       </c>
       <c r="I198">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
@@ -9456,7 +9456,7 @@
         <v>25</v>
       </c>
       <c r="I199">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
@@ -9485,7 +9485,7 @@
         <v>25</v>
       </c>
       <c r="I200">
-        <v>5795</v>
+        <v>6051</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -9543,7 +9543,7 @@
         <v>25</v>
       </c>
       <c r="I202">
-        <v>594</v>
+        <v>611</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
@@ -9572,7 +9572,7 @@
         <v>25</v>
       </c>
       <c r="I203">
-        <v>624</v>
+        <v>613</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>25</v>
       </c>
       <c r="I206">
-        <v>2474</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
@@ -9717,7 +9717,7 @@
         <v>25</v>
       </c>
       <c r="I208">
-        <v>2478</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
@@ -9746,7 +9746,7 @@
         <v>25</v>
       </c>
       <c r="I209">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -9775,7 +9775,7 @@
         <v>25</v>
       </c>
       <c r="I210">
-        <v>5614</v>
+        <v>5685</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -9804,7 +9804,7 @@
         <v>25</v>
       </c>
       <c r="I211">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -9833,7 +9833,7 @@
         <v>25</v>
       </c>
       <c r="I212">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
@@ -9949,7 +9949,7 @@
         <v>25</v>
       </c>
       <c r="I216">
-        <v>3760</v>
+        <v>3742</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
@@ -9978,7 +9978,7 @@
         <v>25</v>
       </c>
       <c r="I217">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
@@ -10036,7 +10036,7 @@
         <v>44</v>
       </c>
       <c r="I219">
-        <v>1543</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
@@ -10065,7 +10065,7 @@
         <v>25</v>
       </c>
       <c r="I220">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
@@ -10094,7 +10094,7 @@
         <v>25</v>
       </c>
       <c r="I221">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
@@ -10123,7 +10123,7 @@
         <v>25</v>
       </c>
       <c r="I222">
-        <v>1523</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
@@ -10239,7 +10239,7 @@
         <v>25</v>
       </c>
       <c r="I226">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>25</v>
       </c>
       <c r="I227">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
@@ -10326,7 +10326,7 @@
         <v>25</v>
       </c>
       <c r="I229">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
@@ -10413,7 +10413,7 @@
         <v>25</v>
       </c>
       <c r="I232">
-        <v>2614</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>25</v>
       </c>
       <c r="I234">
-        <v>3520</v>
+        <v>3487</v>
       </c>
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
@@ -10500,7 +10500,7 @@
         <v>25</v>
       </c>
       <c r="I235">
-        <v>1328</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
@@ -10529,7 +10529,7 @@
         <v>25</v>
       </c>
       <c r="I236">
-        <v>18360</v>
+        <v>17694</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
@@ -10558,7 +10558,7 @@
         <v>25</v>
       </c>
       <c r="I237">
-        <v>46016</v>
+        <v>45765</v>
       </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
@@ -10616,7 +10616,7 @@
         <v>44</v>
       </c>
       <c r="I239">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
@@ -10645,7 +10645,7 @@
         <v>25</v>
       </c>
       <c r="I240">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
@@ -10674,7 +10674,7 @@
         <v>25</v>
       </c>
       <c r="I241">
-        <v>340</v>
+        <v>347</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
@@ -10703,7 +10703,7 @@
         <v>25</v>
       </c>
       <c r="I242">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
@@ -10761,7 +10761,7 @@
         <v>25</v>
       </c>
       <c r="I244">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
@@ -10790,7 +10790,7 @@
         <v>25</v>
       </c>
       <c r="I245">
-        <v>1466</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
@@ -10906,7 +10906,7 @@
         <v>25</v>
       </c>
       <c r="I249">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>993</v>
       </c>
       <c r="B13">
-        <v>46016</v>
+        <v>45765</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -11119,7 +11119,7 @@
         <v>989</v>
       </c>
       <c r="B14">
-        <v>18360</v>
+        <v>17694</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -11127,7 +11127,7 @@
         <v>380</v>
       </c>
       <c r="B15">
-        <v>17040</v>
+        <v>17086</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -11135,7 +11135,7 @@
         <v>669</v>
       </c>
       <c r="B16">
-        <v>12271</v>
+        <v>12264</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>352</v>
       </c>
       <c r="B17">
-        <v>10704</v>
+        <v>9982</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>777</v>
       </c>
       <c r="B18">
-        <v>9478</v>
+        <v>9492</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -11159,7 +11159,7 @@
         <v>201</v>
       </c>
       <c r="B19">
-        <v>9166</v>
+        <v>9270</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -11167,7 +11167,7 @@
         <v>457</v>
       </c>
       <c r="B20">
-        <v>8335</v>
+        <v>8250</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -11175,7 +11175,7 @@
         <v>87</v>
       </c>
       <c r="B21">
-        <v>7540</v>
+        <v>7554</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -11183,7 +11183,7 @@
         <v>497</v>
       </c>
       <c r="B22">
-        <v>7177</v>
+        <v>7336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>